<commit_message>
new feature added for viwe more advanced trakcing
</commit_message>
<xml_diff>
--- a/db/tracker.xlsx
+++ b/db/tracker.xlsx
@@ -400,20 +400,20 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L2"/>
+  <dimension ref="A1:L57"/>
   <cols>
-    <col min="1" max="1" width="14.83203125" customWidth="1"/>
+    <col min="1" max="1" width="43.83203125" customWidth="1"/>
     <col min="2" max="2" width="13.83203125" customWidth="1"/>
-    <col min="3" max="3" width="10.83203125" customWidth="1"/>
+    <col min="3" max="3" width="26.83203125" customWidth="1"/>
     <col min="4" max="4" width="15.83203125" customWidth="1"/>
-    <col min="5" max="5" width="10.83203125" customWidth="1"/>
+    <col min="5" max="5" width="14.83203125" customWidth="1"/>
     <col min="6" max="6" width="10.83203125" customWidth="1"/>
-    <col min="7" max="7" width="10.83203125" customWidth="1"/>
+    <col min="7" max="7" width="13.83203125" customWidth="1"/>
     <col min="8" max="8" width="10.83203125" customWidth="1"/>
     <col min="9" max="9" width="10.83203125" customWidth="1"/>
     <col min="10" max="10" width="10.83203125" customWidth="1"/>
-    <col min="11" max="11" width="10.83203125" customWidth="1"/>
-    <col min="12" max="12" width="10.83203125" customWidth="1"/>
+    <col min="11" max="11" width="13.83203125" customWidth="1"/>
+    <col min="12" max="12" width="13.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -456,19 +456,2142 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>No tasks yet</v>
+        <v>sklearn</v>
+      </c>
+      <c r="B2" t="str">
+        <v/>
+      </c>
+      <c r="C2" t="str">
+        <v>Scikit-Learn/ API</v>
+      </c>
+      <c r="D2" t="str">
+        <v>High</v>
+      </c>
+      <c r="E2" t="str">
+        <v>SPR-2026-W33</v>
+      </c>
+      <c r="F2" t="str">
+        <v>2026-08</v>
+      </c>
+      <c r="G2" t="str">
+        <v>In Progress</v>
+      </c>
+      <c r="H2" t="str">
+        <v>Medium</v>
+      </c>
+      <c r="I2" t="str">
+        <v/>
+      </c>
+      <c r="J2" t="str">
+        <v/>
+      </c>
+      <c r="K2" t="str">
+        <v>Aug 8, 2026</v>
+      </c>
+      <c r="L2" t="str">
+        <v>Aug 8, 2026</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>sklearn.base</v>
+      </c>
+      <c r="B3" t="str">
+        <v/>
+      </c>
+      <c r="C3" t="str">
+        <v>Scikit-Learn/ API</v>
+      </c>
+      <c r="D3" t="str">
+        <v>High</v>
+      </c>
+      <c r="E3" t="str">
+        <v>SPR-2026-W33</v>
+      </c>
+      <c r="F3" t="str">
+        <v>2026-08</v>
+      </c>
+      <c r="G3" t="str">
+        <v>Practice</v>
+      </c>
+      <c r="H3" t="str">
+        <v>Medium</v>
+      </c>
+      <c r="I3" t="str">
+        <v/>
+      </c>
+      <c r="J3" t="str">
+        <v/>
+      </c>
+      <c r="K3" t="str">
+        <v>Aug 8, 2026</v>
+      </c>
+      <c r="L3" t="str">
+        <v>Aug 8, 2026</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>sklearn.calibration</v>
+      </c>
+      <c r="B4" t="str">
+        <v/>
+      </c>
+      <c r="C4" t="str">
+        <v>Scikit-Learn/ API</v>
+      </c>
+      <c r="D4" t="str">
+        <v>High</v>
+      </c>
+      <c r="E4" t="str">
+        <v>SPR-2026-W33</v>
+      </c>
+      <c r="F4" t="str">
+        <v>2026-08</v>
+      </c>
+      <c r="G4" t="str">
+        <v>To Do</v>
+      </c>
+      <c r="H4" t="str">
+        <v>Medium</v>
+      </c>
+      <c r="I4" t="str">
+        <v/>
+      </c>
+      <c r="J4" t="str">
+        <v/>
+      </c>
+      <c r="K4" t="str">
+        <v>Aug 8, 2026</v>
+      </c>
+      <c r="L4" t="str">
+        <v>Aug 8, 2026</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>sklearn.callback</v>
+      </c>
+      <c r="B5" t="str">
+        <v/>
+      </c>
+      <c r="C5" t="str">
+        <v>Scikit-Learn/ API</v>
+      </c>
+      <c r="D5" t="str">
+        <v>High</v>
+      </c>
+      <c r="E5" t="str">
+        <v>SPR-2026-W33</v>
+      </c>
+      <c r="F5" t="str">
+        <v>2026-08</v>
+      </c>
+      <c r="G5" t="str">
+        <v>To Do</v>
+      </c>
+      <c r="H5" t="str">
+        <v>Medium</v>
+      </c>
+      <c r="I5" t="str">
+        <v/>
+      </c>
+      <c r="J5" t="str">
+        <v/>
+      </c>
+      <c r="K5" t="str">
+        <v>Aug 8, 2026</v>
+      </c>
+      <c r="L5" t="str">
+        <v>Aug 8, 2026</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>sklearn.cluster</v>
+      </c>
+      <c r="B6" t="str">
+        <v/>
+      </c>
+      <c r="C6" t="str">
+        <v>Scikit-Learn/ API</v>
+      </c>
+      <c r="D6" t="str">
+        <v>High</v>
+      </c>
+      <c r="E6" t="str">
+        <v>SPR-2026-W33</v>
+      </c>
+      <c r="F6" t="str">
+        <v>2026-08</v>
+      </c>
+      <c r="G6" t="str">
+        <v>To Do</v>
+      </c>
+      <c r="H6" t="str">
+        <v>Medium</v>
+      </c>
+      <c r="I6" t="str">
+        <v/>
+      </c>
+      <c r="J6" t="str">
+        <v/>
+      </c>
+      <c r="K6" t="str">
+        <v>Aug 8, 2026</v>
+      </c>
+      <c r="L6" t="str">
+        <v>Aug 8, 2026</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>sklearn.compose</v>
+      </c>
+      <c r="B7" t="str">
+        <v/>
+      </c>
+      <c r="C7" t="str">
+        <v>Scikit-Learn/ API</v>
+      </c>
+      <c r="D7" t="str">
+        <v>High</v>
+      </c>
+      <c r="E7" t="str">
+        <v>SPR-2026-W33</v>
+      </c>
+      <c r="F7" t="str">
+        <v>2026-08</v>
+      </c>
+      <c r="G7" t="str">
+        <v>To Do</v>
+      </c>
+      <c r="H7" t="str">
+        <v>Medium</v>
+      </c>
+      <c r="I7" t="str">
+        <v/>
+      </c>
+      <c r="J7" t="str">
+        <v/>
+      </c>
+      <c r="K7" t="str">
+        <v>Aug 8, 2026</v>
+      </c>
+      <c r="L7" t="str">
+        <v>Aug 8, 2026</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>sklearn.covariance</v>
+      </c>
+      <c r="B8" t="str">
+        <v/>
+      </c>
+      <c r="C8" t="str">
+        <v>Scikit-Learn/ API</v>
+      </c>
+      <c r="D8" t="str">
+        <v>High</v>
+      </c>
+      <c r="E8" t="str">
+        <v>SPR-2026-W33</v>
+      </c>
+      <c r="F8" t="str">
+        <v>2026-08</v>
+      </c>
+      <c r="G8" t="str">
+        <v>To Do</v>
+      </c>
+      <c r="H8" t="str">
+        <v>Medium</v>
+      </c>
+      <c r="I8" t="str">
+        <v/>
+      </c>
+      <c r="J8" t="str">
+        <v/>
+      </c>
+      <c r="K8" t="str">
+        <v>Aug 8, 2026</v>
+      </c>
+      <c r="L8" t="str">
+        <v>Aug 8, 2026</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>sklearn.cross_decomposition</v>
+      </c>
+      <c r="B9" t="str">
+        <v/>
+      </c>
+      <c r="C9" t="str">
+        <v>Scikit-Learn/ API</v>
+      </c>
+      <c r="D9" t="str">
+        <v>High</v>
+      </c>
+      <c r="E9" t="str">
+        <v>SPR-2026-W33</v>
+      </c>
+      <c r="F9" t="str">
+        <v>2026-08</v>
+      </c>
+      <c r="G9" t="str">
+        <v>To Do</v>
+      </c>
+      <c r="H9" t="str">
+        <v>Medium</v>
+      </c>
+      <c r="I9" t="str">
+        <v/>
+      </c>
+      <c r="J9" t="str">
+        <v/>
+      </c>
+      <c r="K9" t="str">
+        <v>Aug 8, 2026</v>
+      </c>
+      <c r="L9" t="str">
+        <v>Aug 8, 2026</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>sklearn.datasets</v>
+      </c>
+      <c r="B10" t="str">
+        <v/>
+      </c>
+      <c r="C10" t="str">
+        <v>Scikit-Learn/ API</v>
+      </c>
+      <c r="D10" t="str">
+        <v>High</v>
+      </c>
+      <c r="E10" t="str">
+        <v/>
+      </c>
+      <c r="F10" t="str">
+        <v>2026-08</v>
+      </c>
+      <c r="G10" t="str">
+        <v>To Do</v>
+      </c>
+      <c r="H10" t="str">
+        <v>Medium</v>
+      </c>
+      <c r="I10" t="str">
+        <v/>
+      </c>
+      <c r="J10" t="str">
+        <v/>
+      </c>
+      <c r="K10" t="str">
+        <v>Aug 8, 2026</v>
+      </c>
+      <c r="L10" t="str">
+        <v>Aug 8, 2026</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>sklearn.decomposition</v>
+      </c>
+      <c r="B11" t="str">
+        <v/>
+      </c>
+      <c r="C11" t="str">
+        <v>Scikit-Learn/ API</v>
+      </c>
+      <c r="D11" t="str">
+        <v>High</v>
+      </c>
+      <c r="E11" t="str">
+        <v/>
+      </c>
+      <c r="F11" t="str">
+        <v>2026-08</v>
+      </c>
+      <c r="G11" t="str">
+        <v>To Do</v>
+      </c>
+      <c r="H11" t="str">
+        <v>Medium</v>
+      </c>
+      <c r="I11" t="str">
+        <v/>
+      </c>
+      <c r="J11" t="str">
+        <v/>
+      </c>
+      <c r="K11" t="str">
+        <v>Aug 8, 2026</v>
+      </c>
+      <c r="L11" t="str">
+        <v>Aug 8, 2026</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>sklearn.discriminant_analysis</v>
+      </c>
+      <c r="B12" t="str">
+        <v/>
+      </c>
+      <c r="C12" t="str">
+        <v>Scikit-Learn/ API</v>
+      </c>
+      <c r="D12" t="str">
+        <v>High</v>
+      </c>
+      <c r="E12" t="str">
+        <v/>
+      </c>
+      <c r="F12" t="str">
+        <v>2026-08</v>
+      </c>
+      <c r="G12" t="str">
+        <v>To Do</v>
+      </c>
+      <c r="H12" t="str">
+        <v>Medium</v>
+      </c>
+      <c r="I12" t="str">
+        <v/>
+      </c>
+      <c r="J12" t="str">
+        <v/>
+      </c>
+      <c r="K12" t="str">
+        <v>Aug 8, 2026</v>
+      </c>
+      <c r="L12" t="str">
+        <v>Aug 8, 2026</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>sklearn.dummy</v>
+      </c>
+      <c r="B13" t="str">
+        <v/>
+      </c>
+      <c r="C13" t="str">
+        <v>Scikit-Learn/ API</v>
+      </c>
+      <c r="D13" t="str">
+        <v>High</v>
+      </c>
+      <c r="E13" t="str">
+        <v/>
+      </c>
+      <c r="F13" t="str">
+        <v>2026-08</v>
+      </c>
+      <c r="G13" t="str">
+        <v>To Do</v>
+      </c>
+      <c r="H13" t="str">
+        <v>Medium</v>
+      </c>
+      <c r="I13" t="str">
+        <v/>
+      </c>
+      <c r="J13" t="str">
+        <v/>
+      </c>
+      <c r="K13" t="str">
+        <v>Aug 8, 2026</v>
+      </c>
+      <c r="L13" t="str">
+        <v>Aug 8, 2026</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>sklearn.ensemble</v>
+      </c>
+      <c r="B14" t="str">
+        <v/>
+      </c>
+      <c r="C14" t="str">
+        <v>Scikit-Learn/ API</v>
+      </c>
+      <c r="D14" t="str">
+        <v>High</v>
+      </c>
+      <c r="E14" t="str">
+        <v/>
+      </c>
+      <c r="F14" t="str">
+        <v>2026-08</v>
+      </c>
+      <c r="G14" t="str">
+        <v>To Do</v>
+      </c>
+      <c r="H14" t="str">
+        <v>Medium</v>
+      </c>
+      <c r="I14" t="str">
+        <v/>
+      </c>
+      <c r="J14" t="str">
+        <v/>
+      </c>
+      <c r="K14" t="str">
+        <v>Aug 8, 2026</v>
+      </c>
+      <c r="L14" t="str">
+        <v>Aug 8, 2026</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>sklearn.exceptions</v>
+      </c>
+      <c r="B15" t="str">
+        <v/>
+      </c>
+      <c r="C15" t="str">
+        <v>Scikit-Learn/ API</v>
+      </c>
+      <c r="D15" t="str">
+        <v>High</v>
+      </c>
+      <c r="E15" t="str">
+        <v/>
+      </c>
+      <c r="F15" t="str">
+        <v>2026-08</v>
+      </c>
+      <c r="G15" t="str">
+        <v>To Do</v>
+      </c>
+      <c r="H15" t="str">
+        <v>Medium</v>
+      </c>
+      <c r="I15" t="str">
+        <v/>
+      </c>
+      <c r="J15" t="str">
+        <v/>
+      </c>
+      <c r="K15" t="str">
+        <v>Aug 8, 2026</v>
+      </c>
+      <c r="L15" t="str">
+        <v>Aug 8, 2026</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>sklearn.experimental</v>
+      </c>
+      <c r="B16" t="str">
+        <v/>
+      </c>
+      <c r="C16" t="str">
+        <v>Scikit-Learn/ API</v>
+      </c>
+      <c r="D16" t="str">
+        <v>High</v>
+      </c>
+      <c r="E16" t="str">
+        <v/>
+      </c>
+      <c r="F16" t="str">
+        <v>2026-08</v>
+      </c>
+      <c r="G16" t="str">
+        <v>To Do</v>
+      </c>
+      <c r="H16" t="str">
+        <v>Medium</v>
+      </c>
+      <c r="I16" t="str">
+        <v/>
+      </c>
+      <c r="J16" t="str">
+        <v/>
+      </c>
+      <c r="K16" t="str">
+        <v>Aug 8, 2026</v>
+      </c>
+      <c r="L16" t="str">
+        <v>Aug 8, 2026</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>sklearn.feature_extraction</v>
+      </c>
+      <c r="B17" t="str">
+        <v/>
+      </c>
+      <c r="C17" t="str">
+        <v>Scikit-Learn/ API</v>
+      </c>
+      <c r="D17" t="str">
+        <v>High</v>
+      </c>
+      <c r="E17" t="str">
+        <v/>
+      </c>
+      <c r="F17" t="str">
+        <v>2026-08</v>
+      </c>
+      <c r="G17" t="str">
+        <v>To Do</v>
+      </c>
+      <c r="H17" t="str">
+        <v>Medium</v>
+      </c>
+      <c r="I17" t="str">
+        <v/>
+      </c>
+      <c r="J17" t="str">
+        <v/>
+      </c>
+      <c r="K17" t="str">
+        <v>Aug 8, 2026</v>
+      </c>
+      <c r="L17" t="str">
+        <v>Aug 8, 2026</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v>sklearn.feature_selection</v>
+      </c>
+      <c r="B18" t="str">
+        <v/>
+      </c>
+      <c r="C18" t="str">
+        <v>Scikit-Learn/ API</v>
+      </c>
+      <c r="D18" t="str">
+        <v>High</v>
+      </c>
+      <c r="E18" t="str">
+        <v/>
+      </c>
+      <c r="F18" t="str">
+        <v>2026-08</v>
+      </c>
+      <c r="G18" t="str">
+        <v>To Do</v>
+      </c>
+      <c r="H18" t="str">
+        <v>Medium</v>
+      </c>
+      <c r="I18" t="str">
+        <v/>
+      </c>
+      <c r="J18" t="str">
+        <v/>
+      </c>
+      <c r="K18" t="str">
+        <v>Aug 8, 2026</v>
+      </c>
+      <c r="L18" t="str">
+        <v>Aug 8, 2026</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v>sklearn.frozen</v>
+      </c>
+      <c r="B19" t="str">
+        <v/>
+      </c>
+      <c r="C19" t="str">
+        <v>Scikit-Learn/ API</v>
+      </c>
+      <c r="D19" t="str">
+        <v>High</v>
+      </c>
+      <c r="E19" t="str">
+        <v/>
+      </c>
+      <c r="F19" t="str">
+        <v>2026-08</v>
+      </c>
+      <c r="G19" t="str">
+        <v>To Do</v>
+      </c>
+      <c r="H19" t="str">
+        <v>Medium</v>
+      </c>
+      <c r="I19" t="str">
+        <v/>
+      </c>
+      <c r="J19" t="str">
+        <v/>
+      </c>
+      <c r="K19" t="str">
+        <v>Aug 8, 2026</v>
+      </c>
+      <c r="L19" t="str">
+        <v>Aug 8, 2026</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <v>sklearn.gaussian_process</v>
+      </c>
+      <c r="B20" t="str">
+        <v/>
+      </c>
+      <c r="C20" t="str">
+        <v>Scikit-Learn/ API</v>
+      </c>
+      <c r="D20" t="str">
+        <v>High</v>
+      </c>
+      <c r="E20" t="str">
+        <v/>
+      </c>
+      <c r="F20" t="str">
+        <v>2026-08</v>
+      </c>
+      <c r="G20" t="str">
+        <v>To Do</v>
+      </c>
+      <c r="H20" t="str">
+        <v>Medium</v>
+      </c>
+      <c r="I20" t="str">
+        <v/>
+      </c>
+      <c r="J20" t="str">
+        <v/>
+      </c>
+      <c r="K20" t="str">
+        <v>Aug 8, 2026</v>
+      </c>
+      <c r="L20" t="str">
+        <v>Aug 8, 2026</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="str">
+        <v>sklearn.impute</v>
+      </c>
+      <c r="B21" t="str">
+        <v/>
+      </c>
+      <c r="C21" t="str">
+        <v>Scikit-Learn/ API</v>
+      </c>
+      <c r="D21" t="str">
+        <v>High</v>
+      </c>
+      <c r="E21" t="str">
+        <v/>
+      </c>
+      <c r="F21" t="str">
+        <v>2026-08</v>
+      </c>
+      <c r="G21" t="str">
+        <v>To Do</v>
+      </c>
+      <c r="H21" t="str">
+        <v>Medium</v>
+      </c>
+      <c r="I21" t="str">
+        <v/>
+      </c>
+      <c r="J21" t="str">
+        <v/>
+      </c>
+      <c r="K21" t="str">
+        <v>Aug 8, 2026</v>
+      </c>
+      <c r="L21" t="str">
+        <v>Aug 8, 2026</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="str">
+        <v>sklearn.inspection</v>
+      </c>
+      <c r="B22" t="str">
+        <v/>
+      </c>
+      <c r="C22" t="str">
+        <v>Scikit-Learn/ API</v>
+      </c>
+      <c r="D22" t="str">
+        <v>High</v>
+      </c>
+      <c r="E22" t="str">
+        <v/>
+      </c>
+      <c r="F22" t="str">
+        <v>2026-08</v>
+      </c>
+      <c r="G22" t="str">
+        <v>To Do</v>
+      </c>
+      <c r="H22" t="str">
+        <v>Medium</v>
+      </c>
+      <c r="I22" t="str">
+        <v/>
+      </c>
+      <c r="J22" t="str">
+        <v/>
+      </c>
+      <c r="K22" t="str">
+        <v>Aug 8, 2026</v>
+      </c>
+      <c r="L22" t="str">
+        <v>Aug 8, 2026</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="str">
+        <v>sklearn.isotonic</v>
+      </c>
+      <c r="B23" t="str">
+        <v/>
+      </c>
+      <c r="C23" t="str">
+        <v>Scikit-Learn/ API</v>
+      </c>
+      <c r="D23" t="str">
+        <v>High</v>
+      </c>
+      <c r="E23" t="str">
+        <v/>
+      </c>
+      <c r="F23" t="str">
+        <v>2026-08</v>
+      </c>
+      <c r="G23" t="str">
+        <v>To Do</v>
+      </c>
+      <c r="H23" t="str">
+        <v>Medium</v>
+      </c>
+      <c r="I23" t="str">
+        <v/>
+      </c>
+      <c r="J23" t="str">
+        <v/>
+      </c>
+      <c r="K23" t="str">
+        <v>Aug 8, 2026</v>
+      </c>
+      <c r="L23" t="str">
+        <v>Aug 8, 2026</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="str">
+        <v>sklearn.kernel_approximation</v>
+      </c>
+      <c r="B24" t="str">
+        <v/>
+      </c>
+      <c r="C24" t="str">
+        <v>Scikit-Learn/ API</v>
+      </c>
+      <c r="D24" t="str">
+        <v>High</v>
+      </c>
+      <c r="E24" t="str">
+        <v/>
+      </c>
+      <c r="F24" t="str">
+        <v>2026-08</v>
+      </c>
+      <c r="G24" t="str">
+        <v>To Do</v>
+      </c>
+      <c r="H24" t="str">
+        <v>Medium</v>
+      </c>
+      <c r="I24" t="str">
+        <v/>
+      </c>
+      <c r="J24" t="str">
+        <v/>
+      </c>
+      <c r="K24" t="str">
+        <v>Aug 8, 2026</v>
+      </c>
+      <c r="L24" t="str">
+        <v>Aug 8, 2026</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="str">
+        <v>sklearn.kernel_ridge</v>
+      </c>
+      <c r="B25" t="str">
+        <v/>
+      </c>
+      <c r="C25" t="str">
+        <v>Scikit-Learn/ API</v>
+      </c>
+      <c r="D25" t="str">
+        <v>High</v>
+      </c>
+      <c r="E25" t="str">
+        <v/>
+      </c>
+      <c r="F25" t="str">
+        <v>2026-08</v>
+      </c>
+      <c r="G25" t="str">
+        <v>To Do</v>
+      </c>
+      <c r="H25" t="str">
+        <v>Medium</v>
+      </c>
+      <c r="I25" t="str">
+        <v/>
+      </c>
+      <c r="J25" t="str">
+        <v/>
+      </c>
+      <c r="K25" t="str">
+        <v>Aug 8, 2026</v>
+      </c>
+      <c r="L25" t="str">
+        <v>Aug 8, 2026</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="str">
+        <v>sklearn.linear_model</v>
+      </c>
+      <c r="B26" t="str">
+        <v/>
+      </c>
+      <c r="C26" t="str">
+        <v>Scikit-Learn/ API</v>
+      </c>
+      <c r="D26" t="str">
+        <v>High</v>
+      </c>
+      <c r="E26" t="str">
+        <v/>
+      </c>
+      <c r="F26" t="str">
+        <v>2026-08</v>
+      </c>
+      <c r="G26" t="str">
+        <v>To Do</v>
+      </c>
+      <c r="H26" t="str">
+        <v>Medium</v>
+      </c>
+      <c r="I26" t="str">
+        <v/>
+      </c>
+      <c r="J26" t="str">
+        <v/>
+      </c>
+      <c r="K26" t="str">
+        <v>Aug 8, 2026</v>
+      </c>
+      <c r="L26" t="str">
+        <v>Aug 8, 2026</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="str">
+        <v>sklearn.manifold</v>
+      </c>
+      <c r="B27" t="str">
+        <v/>
+      </c>
+      <c r="C27" t="str">
+        <v>Scikit-Learn/ API</v>
+      </c>
+      <c r="D27" t="str">
+        <v>High</v>
+      </c>
+      <c r="E27" t="str">
+        <v/>
+      </c>
+      <c r="F27" t="str">
+        <v>2026-08</v>
+      </c>
+      <c r="G27" t="str">
+        <v>To Do</v>
+      </c>
+      <c r="H27" t="str">
+        <v>Medium</v>
+      </c>
+      <c r="I27" t="str">
+        <v/>
+      </c>
+      <c r="J27" t="str">
+        <v/>
+      </c>
+      <c r="K27" t="str">
+        <v>Aug 8, 2026</v>
+      </c>
+      <c r="L27" t="str">
+        <v>Aug 8, 2026</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="str">
+        <v>sklearn.metrics</v>
+      </c>
+      <c r="B28" t="str">
+        <v/>
+      </c>
+      <c r="C28" t="str">
+        <v>Scikit-Learn/ API</v>
+      </c>
+      <c r="D28" t="str">
+        <v>High</v>
+      </c>
+      <c r="E28" t="str">
+        <v/>
+      </c>
+      <c r="F28" t="str">
+        <v>2026-08</v>
+      </c>
+      <c r="G28" t="str">
+        <v>To Do</v>
+      </c>
+      <c r="H28" t="str">
+        <v>Medium</v>
+      </c>
+      <c r="I28" t="str">
+        <v/>
+      </c>
+      <c r="J28" t="str">
+        <v/>
+      </c>
+      <c r="K28" t="str">
+        <v>Aug 8, 2026</v>
+      </c>
+      <c r="L28" t="str">
+        <v>Aug 8, 2026</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="str">
+        <v>sklearn.mixture</v>
+      </c>
+      <c r="B29" t="str">
+        <v/>
+      </c>
+      <c r="C29" t="str">
+        <v>Scikit-Learn/ API</v>
+      </c>
+      <c r="D29" t="str">
+        <v>High</v>
+      </c>
+      <c r="E29" t="str">
+        <v/>
+      </c>
+      <c r="F29" t="str">
+        <v>2026-08</v>
+      </c>
+      <c r="G29" t="str">
+        <v>To Do</v>
+      </c>
+      <c r="H29" t="str">
+        <v>Medium</v>
+      </c>
+      <c r="I29" t="str">
+        <v/>
+      </c>
+      <c r="J29" t="str">
+        <v/>
+      </c>
+      <c r="K29" t="str">
+        <v>Aug 8, 2026</v>
+      </c>
+      <c r="L29" t="str">
+        <v>Aug 8, 2026</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="str">
+        <v>sklearn.model_selection</v>
+      </c>
+      <c r="B30" t="str">
+        <v/>
+      </c>
+      <c r="C30" t="str">
+        <v>Scikit-Learn/ API</v>
+      </c>
+      <c r="D30" t="str">
+        <v>High</v>
+      </c>
+      <c r="E30" t="str">
+        <v/>
+      </c>
+      <c r="F30" t="str">
+        <v>2026-08</v>
+      </c>
+      <c r="G30" t="str">
+        <v>To Do</v>
+      </c>
+      <c r="H30" t="str">
+        <v>Medium</v>
+      </c>
+      <c r="I30" t="str">
+        <v/>
+      </c>
+      <c r="J30" t="str">
+        <v/>
+      </c>
+      <c r="K30" t="str">
+        <v>Aug 8, 2026</v>
+      </c>
+      <c r="L30" t="str">
+        <v>Aug 8, 2026</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="str">
+        <v>sklearn.multiclass</v>
+      </c>
+      <c r="B31" t="str">
+        <v/>
+      </c>
+      <c r="C31" t="str">
+        <v>Scikit-Learn/ API</v>
+      </c>
+      <c r="D31" t="str">
+        <v>High</v>
+      </c>
+      <c r="E31" t="str">
+        <v/>
+      </c>
+      <c r="F31" t="str">
+        <v>2026-08</v>
+      </c>
+      <c r="G31" t="str">
+        <v>To Do</v>
+      </c>
+      <c r="H31" t="str">
+        <v>Medium</v>
+      </c>
+      <c r="I31" t="str">
+        <v/>
+      </c>
+      <c r="J31" t="str">
+        <v/>
+      </c>
+      <c r="K31" t="str">
+        <v>Aug 8, 2026</v>
+      </c>
+      <c r="L31" t="str">
+        <v>Aug 8, 2026</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="str">
+        <v>sklearn.multioutput</v>
+      </c>
+      <c r="B32" t="str">
+        <v/>
+      </c>
+      <c r="C32" t="str">
+        <v>Scikit-Learn/ API</v>
+      </c>
+      <c r="D32" t="str">
+        <v>High</v>
+      </c>
+      <c r="E32" t="str">
+        <v/>
+      </c>
+      <c r="F32" t="str">
+        <v>2026-08</v>
+      </c>
+      <c r="G32" t="str">
+        <v>To Do</v>
+      </c>
+      <c r="H32" t="str">
+        <v>Medium</v>
+      </c>
+      <c r="I32" t="str">
+        <v/>
+      </c>
+      <c r="J32" t="str">
+        <v/>
+      </c>
+      <c r="K32" t="str">
+        <v>Aug 8, 2026</v>
+      </c>
+      <c r="L32" t="str">
+        <v>Aug 8, 2026</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="str">
+        <v>sklearn.naive_bayes</v>
+      </c>
+      <c r="B33" t="str">
+        <v/>
+      </c>
+      <c r="C33" t="str">
+        <v>Scikit-Learn/ API</v>
+      </c>
+      <c r="D33" t="str">
+        <v>High</v>
+      </c>
+      <c r="E33" t="str">
+        <v/>
+      </c>
+      <c r="F33" t="str">
+        <v>2026-08</v>
+      </c>
+      <c r="G33" t="str">
+        <v>To Do</v>
+      </c>
+      <c r="H33" t="str">
+        <v>Medium</v>
+      </c>
+      <c r="I33" t="str">
+        <v/>
+      </c>
+      <c r="J33" t="str">
+        <v/>
+      </c>
+      <c r="K33" t="str">
+        <v>Aug 8, 2026</v>
+      </c>
+      <c r="L33" t="str">
+        <v>Aug 8, 2026</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="str">
+        <v>sklearn.neighbors</v>
+      </c>
+      <c r="B34" t="str">
+        <v/>
+      </c>
+      <c r="C34" t="str">
+        <v>Scikit-Learn/ API</v>
+      </c>
+      <c r="D34" t="str">
+        <v>High</v>
+      </c>
+      <c r="E34" t="str">
+        <v/>
+      </c>
+      <c r="F34" t="str">
+        <v>2026-08</v>
+      </c>
+      <c r="G34" t="str">
+        <v>To Do</v>
+      </c>
+      <c r="H34" t="str">
+        <v>Medium</v>
+      </c>
+      <c r="I34" t="str">
+        <v/>
+      </c>
+      <c r="J34" t="str">
+        <v/>
+      </c>
+      <c r="K34" t="str">
+        <v>Aug 8, 2026</v>
+      </c>
+      <c r="L34" t="str">
+        <v>Aug 8, 2026</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="str">
+        <v>sklearn.neural_network</v>
+      </c>
+      <c r="B35" t="str">
+        <v/>
+      </c>
+      <c r="C35" t="str">
+        <v>Scikit-Learn/ API</v>
+      </c>
+      <c r="D35" t="str">
+        <v>High</v>
+      </c>
+      <c r="E35" t="str">
+        <v/>
+      </c>
+      <c r="F35" t="str">
+        <v>2026-08</v>
+      </c>
+      <c r="G35" t="str">
+        <v>To Do</v>
+      </c>
+      <c r="H35" t="str">
+        <v>Medium</v>
+      </c>
+      <c r="I35" t="str">
+        <v/>
+      </c>
+      <c r="J35" t="str">
+        <v/>
+      </c>
+      <c r="K35" t="str">
+        <v>Aug 8, 2026</v>
+      </c>
+      <c r="L35" t="str">
+        <v>Aug 8, 2026</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="str">
+        <v>sklearn.pipeline</v>
+      </c>
+      <c r="B36" t="str">
+        <v/>
+      </c>
+      <c r="C36" t="str">
+        <v>Scikit-Learn/ API</v>
+      </c>
+      <c r="D36" t="str">
+        <v>High</v>
+      </c>
+      <c r="E36" t="str">
+        <v/>
+      </c>
+      <c r="F36" t="str">
+        <v>2026-08</v>
+      </c>
+      <c r="G36" t="str">
+        <v>To Do</v>
+      </c>
+      <c r="H36" t="str">
+        <v>Medium</v>
+      </c>
+      <c r="I36" t="str">
+        <v/>
+      </c>
+      <c r="J36" t="str">
+        <v/>
+      </c>
+      <c r="K36" t="str">
+        <v>Aug 8, 2026</v>
+      </c>
+      <c r="L36" t="str">
+        <v>Aug 8, 2026</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="str">
+        <v>sklearn.preprocessing</v>
+      </c>
+      <c r="B37" t="str">
+        <v/>
+      </c>
+      <c r="C37" t="str">
+        <v>Scikit-Learn/ API</v>
+      </c>
+      <c r="D37" t="str">
+        <v>High</v>
+      </c>
+      <c r="E37" t="str">
+        <v/>
+      </c>
+      <c r="F37" t="str">
+        <v>2026-08</v>
+      </c>
+      <c r="G37" t="str">
+        <v>To Do</v>
+      </c>
+      <c r="H37" t="str">
+        <v>Medium</v>
+      </c>
+      <c r="I37" t="str">
+        <v/>
+      </c>
+      <c r="J37" t="str">
+        <v/>
+      </c>
+      <c r="K37" t="str">
+        <v>Aug 8, 2026</v>
+      </c>
+      <c r="L37" t="str">
+        <v>Aug 8, 2026</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="str">
+        <v>sklearn.random_projection</v>
+      </c>
+      <c r="B38" t="str">
+        <v/>
+      </c>
+      <c r="C38" t="str">
+        <v>Scikit-Learn/ API</v>
+      </c>
+      <c r="D38" t="str">
+        <v>High</v>
+      </c>
+      <c r="E38" t="str">
+        <v/>
+      </c>
+      <c r="F38" t="str">
+        <v>2026-08</v>
+      </c>
+      <c r="G38" t="str">
+        <v>To Do</v>
+      </c>
+      <c r="H38" t="str">
+        <v>Medium</v>
+      </c>
+      <c r="I38" t="str">
+        <v/>
+      </c>
+      <c r="J38" t="str">
+        <v/>
+      </c>
+      <c r="K38" t="str">
+        <v>Aug 8, 2026</v>
+      </c>
+      <c r="L38" t="str">
+        <v>Aug 8, 2026</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="str">
+        <v>sklearn.semi_supervised</v>
+      </c>
+      <c r="B39" t="str">
+        <v/>
+      </c>
+      <c r="C39" t="str">
+        <v>Scikit-Learn/ API</v>
+      </c>
+      <c r="D39" t="str">
+        <v>High</v>
+      </c>
+      <c r="E39" t="str">
+        <v/>
+      </c>
+      <c r="F39" t="str">
+        <v>2026-08</v>
+      </c>
+      <c r="G39" t="str">
+        <v>To Do</v>
+      </c>
+      <c r="H39" t="str">
+        <v>Medium</v>
+      </c>
+      <c r="I39" t="str">
+        <v/>
+      </c>
+      <c r="J39" t="str">
+        <v/>
+      </c>
+      <c r="K39" t="str">
+        <v>Aug 8, 2026</v>
+      </c>
+      <c r="L39" t="str">
+        <v>Aug 8, 2026</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="str">
+        <v>sklearn.svm</v>
+      </c>
+      <c r="B40" t="str">
+        <v/>
+      </c>
+      <c r="C40" t="str">
+        <v>Scikit-Learn/ API</v>
+      </c>
+      <c r="D40" t="str">
+        <v>High</v>
+      </c>
+      <c r="E40" t="str">
+        <v/>
+      </c>
+      <c r="F40" t="str">
+        <v>2026-08</v>
+      </c>
+      <c r="G40" t="str">
+        <v>To Do</v>
+      </c>
+      <c r="H40" t="str">
+        <v>Medium</v>
+      </c>
+      <c r="I40" t="str">
+        <v/>
+      </c>
+      <c r="J40" t="str">
+        <v/>
+      </c>
+      <c r="K40" t="str">
+        <v>Aug 8, 2026</v>
+      </c>
+      <c r="L40" t="str">
+        <v>Aug 8, 2026</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="str">
+        <v>sklearn.tree</v>
+      </c>
+      <c r="B41" t="str">
+        <v/>
+      </c>
+      <c r="C41" t="str">
+        <v>Scikit-Learn/ API</v>
+      </c>
+      <c r="D41" t="str">
+        <v>High</v>
+      </c>
+      <c r="E41" t="str">
+        <v/>
+      </c>
+      <c r="F41" t="str">
+        <v>2026-08</v>
+      </c>
+      <c r="G41" t="str">
+        <v>To Do</v>
+      </c>
+      <c r="H41" t="str">
+        <v>Medium</v>
+      </c>
+      <c r="I41" t="str">
+        <v/>
+      </c>
+      <c r="J41" t="str">
+        <v/>
+      </c>
+      <c r="K41" t="str">
+        <v>Aug 8, 2026</v>
+      </c>
+      <c r="L41" t="str">
+        <v>Aug 8, 2026</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="str">
+        <v>sklearn.utils</v>
+      </c>
+      <c r="B42" t="str">
+        <v/>
+      </c>
+      <c r="C42" t="str">
+        <v>Scikit-Learn/ API</v>
+      </c>
+      <c r="D42" t="str">
+        <v>High</v>
+      </c>
+      <c r="E42" t="str">
+        <v/>
+      </c>
+      <c r="F42" t="str">
+        <v>2026-08</v>
+      </c>
+      <c r="G42" t="str">
+        <v>To Do</v>
+      </c>
+      <c r="H42" t="str">
+        <v>Medium</v>
+      </c>
+      <c r="I42" t="str">
+        <v/>
+      </c>
+      <c r="J42" t="str">
+        <v/>
+      </c>
+      <c r="K42" t="str">
+        <v>Aug 8, 2026</v>
+      </c>
+      <c r="L42" t="str">
+        <v>Aug 8, 2026</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="str">
+        <v>Supervised learning</v>
+      </c>
+      <c r="B43" t="str">
+        <v/>
+      </c>
+      <c r="C43" t="str">
+        <v>Scikit-Learn/ User Guide</v>
+      </c>
+      <c r="D43" t="str">
+        <v>High</v>
+      </c>
+      <c r="E43" t="str">
+        <v/>
+      </c>
+      <c r="F43" t="str">
+        <v>2026-08</v>
+      </c>
+      <c r="G43" t="str">
+        <v>To Do</v>
+      </c>
+      <c r="H43" t="str">
+        <v>Medium</v>
+      </c>
+      <c r="I43" t="str">
+        <v/>
+      </c>
+      <c r="J43" t="str">
+        <v/>
+      </c>
+      <c r="K43" t="str">
+        <v>Aug 8, 2026</v>
+      </c>
+      <c r="L43" t="str">
+        <v>Aug 8, 2026</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="str">
+        <v>Unsupervised learning</v>
+      </c>
+      <c r="B44" t="str">
+        <v/>
+      </c>
+      <c r="C44" t="str">
+        <v>Scikit-Learn/ User Guide</v>
+      </c>
+      <c r="D44" t="str">
+        <v>High</v>
+      </c>
+      <c r="E44" t="str">
+        <v/>
+      </c>
+      <c r="F44" t="str">
+        <v>2026-08</v>
+      </c>
+      <c r="G44" t="str">
+        <v>To Do</v>
+      </c>
+      <c r="H44" t="str">
+        <v>Medium</v>
+      </c>
+      <c r="I44" t="str">
+        <v/>
+      </c>
+      <c r="J44" t="str">
+        <v/>
+      </c>
+      <c r="K44" t="str">
+        <v>Aug 8, 2026</v>
+      </c>
+      <c r="L44" t="str">
+        <v>Aug 8, 2026</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="str">
+        <v>Model selection and evaluation</v>
+      </c>
+      <c r="B45" t="str">
+        <v/>
+      </c>
+      <c r="C45" t="str">
+        <v>Scikit-Learn/ User Guide</v>
+      </c>
+      <c r="D45" t="str">
+        <v>High</v>
+      </c>
+      <c r="E45" t="str">
+        <v/>
+      </c>
+      <c r="F45" t="str">
+        <v>2026-08</v>
+      </c>
+      <c r="G45" t="str">
+        <v>To Do</v>
+      </c>
+      <c r="H45" t="str">
+        <v>Medium</v>
+      </c>
+      <c r="I45" t="str">
+        <v/>
+      </c>
+      <c r="J45" t="str">
+        <v/>
+      </c>
+      <c r="K45" t="str">
+        <v>Aug 8, 2026</v>
+      </c>
+      <c r="L45" t="str">
+        <v>Aug 8, 2026</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="str">
+        <v>Metadata Routing</v>
+      </c>
+      <c r="B46" t="str">
+        <v/>
+      </c>
+      <c r="C46" t="str">
+        <v>Scikit-Learn/ User Guide</v>
+      </c>
+      <c r="D46" t="str">
+        <v>High</v>
+      </c>
+      <c r="E46" t="str">
+        <v/>
+      </c>
+      <c r="F46" t="str">
+        <v>2026-08</v>
+      </c>
+      <c r="G46" t="str">
+        <v>To Do</v>
+      </c>
+      <c r="H46" t="str">
+        <v>Medium</v>
+      </c>
+      <c r="I46" t="str">
+        <v/>
+      </c>
+      <c r="J46" t="str">
+        <v/>
+      </c>
+      <c r="K46" t="str">
+        <v>Aug 8, 2026</v>
+      </c>
+      <c r="L46" t="str">
+        <v>Aug 8, 2026</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="str">
+        <v>Inspection</v>
+      </c>
+      <c r="B47" t="str">
+        <v/>
+      </c>
+      <c r="C47" t="str">
+        <v>Scikit-Learn/ User Guide</v>
+      </c>
+      <c r="D47" t="str">
+        <v>High</v>
+      </c>
+      <c r="E47" t="str">
+        <v/>
+      </c>
+      <c r="F47" t="str">
+        <v>2026-08</v>
+      </c>
+      <c r="G47" t="str">
+        <v>To Do</v>
+      </c>
+      <c r="H47" t="str">
+        <v>Medium</v>
+      </c>
+      <c r="I47" t="str">
+        <v/>
+      </c>
+      <c r="J47" t="str">
+        <v/>
+      </c>
+      <c r="K47" t="str">
+        <v>Aug 8, 2026</v>
+      </c>
+      <c r="L47" t="str">
+        <v>Aug 8, 2026</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="str">
+        <v>Visualizations</v>
+      </c>
+      <c r="B48" t="str">
+        <v/>
+      </c>
+      <c r="C48" t="str">
+        <v>Scikit-Learn/ User Guide</v>
+      </c>
+      <c r="D48" t="str">
+        <v>High</v>
+      </c>
+      <c r="E48" t="str">
+        <v/>
+      </c>
+      <c r="F48" t="str">
+        <v>2026-08</v>
+      </c>
+      <c r="G48" t="str">
+        <v>To Do</v>
+      </c>
+      <c r="H48" t="str">
+        <v>Medium</v>
+      </c>
+      <c r="I48" t="str">
+        <v/>
+      </c>
+      <c r="J48" t="str">
+        <v/>
+      </c>
+      <c r="K48" t="str">
+        <v>Aug 8, 2026</v>
+      </c>
+      <c r="L48" t="str">
+        <v>Aug 8, 2026</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="str">
+        <v>Callbacks</v>
+      </c>
+      <c r="B49" t="str">
+        <v/>
+      </c>
+      <c r="C49" t="str">
+        <v>Scikit-Learn/ User Guide</v>
+      </c>
+      <c r="D49" t="str">
+        <v>High</v>
+      </c>
+      <c r="E49" t="str">
+        <v/>
+      </c>
+      <c r="F49" t="str">
+        <v>2026-08</v>
+      </c>
+      <c r="G49" t="str">
+        <v>To Do</v>
+      </c>
+      <c r="H49" t="str">
+        <v>Medium</v>
+      </c>
+      <c r="I49" t="str">
+        <v/>
+      </c>
+      <c r="J49" t="str">
+        <v/>
+      </c>
+      <c r="K49" t="str">
+        <v>Aug 8, 2026</v>
+      </c>
+      <c r="L49" t="str">
+        <v>Aug 8, 2026</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="str">
+        <v>Dataset transformations</v>
+      </c>
+      <c r="B50" t="str">
+        <v/>
+      </c>
+      <c r="C50" t="str">
+        <v>Scikit-Learn/ User Guide</v>
+      </c>
+      <c r="D50" t="str">
+        <v>High</v>
+      </c>
+      <c r="E50" t="str">
+        <v/>
+      </c>
+      <c r="F50" t="str">
+        <v>2026-08</v>
+      </c>
+      <c r="G50" t="str">
+        <v>To Do</v>
+      </c>
+      <c r="H50" t="str">
+        <v>Medium</v>
+      </c>
+      <c r="I50" t="str">
+        <v/>
+      </c>
+      <c r="J50" t="str">
+        <v/>
+      </c>
+      <c r="K50" t="str">
+        <v>Aug 8, 2026</v>
+      </c>
+      <c r="L50" t="str">
+        <v>Aug 8, 2026</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="str">
+        <v>Dataset loading utilities</v>
+      </c>
+      <c r="B51" t="str">
+        <v/>
+      </c>
+      <c r="C51" t="str">
+        <v>Scikit-Learn/ User Guide</v>
+      </c>
+      <c r="D51" t="str">
+        <v>High</v>
+      </c>
+      <c r="E51" t="str">
+        <v/>
+      </c>
+      <c r="F51" t="str">
+        <v>2026-08</v>
+      </c>
+      <c r="G51" t="str">
+        <v>To Do</v>
+      </c>
+      <c r="H51" t="str">
+        <v>Medium</v>
+      </c>
+      <c r="I51" t="str">
+        <v/>
+      </c>
+      <c r="J51" t="str">
+        <v/>
+      </c>
+      <c r="K51" t="str">
+        <v>Aug 8, 2026</v>
+      </c>
+      <c r="L51" t="str">
+        <v>Aug 8, 2026</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="str">
+        <v>Computing with scikit-learn</v>
+      </c>
+      <c r="B52" t="str">
+        <v/>
+      </c>
+      <c r="C52" t="str">
+        <v>Scikit-Learn/ User Guide</v>
+      </c>
+      <c r="D52" t="str">
+        <v>High</v>
+      </c>
+      <c r="E52" t="str">
+        <v/>
+      </c>
+      <c r="F52" t="str">
+        <v>2026-08</v>
+      </c>
+      <c r="G52" t="str">
+        <v>To Do</v>
+      </c>
+      <c r="H52" t="str">
+        <v>Medium</v>
+      </c>
+      <c r="I52" t="str">
+        <v/>
+      </c>
+      <c r="J52" t="str">
+        <v/>
+      </c>
+      <c r="K52" t="str">
+        <v>Aug 8, 2026</v>
+      </c>
+      <c r="L52" t="str">
+        <v>Aug 8, 2026</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="str">
+        <v>Model persistence</v>
+      </c>
+      <c r="B53" t="str">
+        <v/>
+      </c>
+      <c r="C53" t="str">
+        <v>Scikit-Learn/ User Guide</v>
+      </c>
+      <c r="D53" t="str">
+        <v>High</v>
+      </c>
+      <c r="E53" t="str">
+        <v/>
+      </c>
+      <c r="F53" t="str">
+        <v>2026-08</v>
+      </c>
+      <c r="G53" t="str">
+        <v>To Do</v>
+      </c>
+      <c r="H53" t="str">
+        <v>Medium</v>
+      </c>
+      <c r="I53" t="str">
+        <v/>
+      </c>
+      <c r="J53" t="str">
+        <v/>
+      </c>
+      <c r="K53" t="str">
+        <v>Aug 8, 2026</v>
+      </c>
+      <c r="L53" t="str">
+        <v>Aug 8, 2026</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="str">
+        <v>Common pitfalls and recommended practices</v>
+      </c>
+      <c r="B54" t="str">
+        <v/>
+      </c>
+      <c r="C54" t="str">
+        <v>Scikit-Learn/ User Guide</v>
+      </c>
+      <c r="D54" t="str">
+        <v>High</v>
+      </c>
+      <c r="E54" t="str">
+        <v/>
+      </c>
+      <c r="F54" t="str">
+        <v>2026-08</v>
+      </c>
+      <c r="G54" t="str">
+        <v>To Do</v>
+      </c>
+      <c r="H54" t="str">
+        <v>Medium</v>
+      </c>
+      <c r="I54" t="str">
+        <v/>
+      </c>
+      <c r="J54" t="str">
+        <v/>
+      </c>
+      <c r="K54" t="str">
+        <v>Aug 8, 2026</v>
+      </c>
+      <c r="L54" t="str">
+        <v>Aug 8, 2026</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="str">
+        <v>Data Interoperability</v>
+      </c>
+      <c r="B55" t="str">
+        <v/>
+      </c>
+      <c r="C55" t="str">
+        <v>Scikit-Learn/ User Guide</v>
+      </c>
+      <c r="D55" t="str">
+        <v>High</v>
+      </c>
+      <c r="E55" t="str">
+        <v/>
+      </c>
+      <c r="F55" t="str">
+        <v>2026-08</v>
+      </c>
+      <c r="G55" t="str">
+        <v>To Do</v>
+      </c>
+      <c r="H55" t="str">
+        <v>Medium</v>
+      </c>
+      <c r="I55" t="str">
+        <v/>
+      </c>
+      <c r="J55" t="str">
+        <v/>
+      </c>
+      <c r="K55" t="str">
+        <v>Aug 8, 2026</v>
+      </c>
+      <c r="L55" t="str">
+        <v>Aug 8, 2026</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="str">
+        <v>Choosing the right estimator</v>
+      </c>
+      <c r="B56" t="str">
+        <v/>
+      </c>
+      <c r="C56" t="str">
+        <v>Scikit-Learn/ User Guide</v>
+      </c>
+      <c r="D56" t="str">
+        <v>High</v>
+      </c>
+      <c r="E56" t="str">
+        <v/>
+      </c>
+      <c r="F56" t="str">
+        <v>2026-08</v>
+      </c>
+      <c r="G56" t="str">
+        <v>To Do</v>
+      </c>
+      <c r="H56" t="str">
+        <v>Medium</v>
+      </c>
+      <c r="I56" t="str">
+        <v/>
+      </c>
+      <c r="J56" t="str">
+        <v/>
+      </c>
+      <c r="K56" t="str">
+        <v>Aug 8, 2026</v>
+      </c>
+      <c r="L56" t="str">
+        <v>Aug 8, 2026</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="str">
+        <v>External Resources, Videos and Talks</v>
+      </c>
+      <c r="B57" t="str">
+        <v/>
+      </c>
+      <c r="C57" t="str">
+        <v>Scikit-Learn/ User Guide</v>
+      </c>
+      <c r="D57" t="str">
+        <v>High</v>
+      </c>
+      <c r="E57" t="str">
+        <v/>
+      </c>
+      <c r="F57" t="str">
+        <v>2026-08</v>
+      </c>
+      <c r="G57" t="str">
+        <v>To Do</v>
+      </c>
+      <c r="H57" t="str">
+        <v>Medium</v>
+      </c>
+      <c r="I57" t="str">
+        <v/>
+      </c>
+      <c r="J57" t="str">
+        <v/>
+      </c>
+      <c r="K57" t="str">
+        <v>Aug 8, 2026</v>
+      </c>
+      <c r="L57" t="str">
+        <v>Aug 8, 2026</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:L2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:L57"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L2"/>
+  <dimension ref="A1:L3"/>
   <cols>
     <col min="1" max="1" width="14.83203125" customWidth="1"/>
     <col min="2" max="2" width="10.83203125" customWidth="1"/>
@@ -560,18 +2683,56 @@
         <v>0%</v>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>SPR-2026-W33</v>
+      </c>
+      <c r="B3" t="str">
+        <v/>
+      </c>
+      <c r="C3" t="str">
+        <v>2026-08-09</v>
+      </c>
+      <c r="D3" t="str">
+        <v>2026-08-14</v>
+      </c>
+      <c r="E3" t="str">
+        <v>2026-08</v>
+      </c>
+      <c r="F3">
+        <v>8</v>
+      </c>
+      <c r="G3">
+        <v>0</v>
+      </c>
+      <c r="H3">
+        <v>1</v>
+      </c>
+      <c r="I3">
+        <v>1</v>
+      </c>
+      <c r="J3">
+        <v>0</v>
+      </c>
+      <c r="K3">
+        <v>6</v>
+      </c>
+      <c r="L3" t="str">
+        <v>0%</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:L2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:L3"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K2"/>
+  <dimension ref="A1:K3"/>
   <cols>
-    <col min="1" max="1" width="14.83203125" customWidth="1"/>
+    <col min="1" max="1" width="26.83203125" customWidth="1"/>
     <col min="2" max="2" width="13.83203125" customWidth="1"/>
     <col min="3" max="3" width="10.83203125" customWidth="1"/>
     <col min="4" max="4" width="13.83203125" customWidth="1"/>
@@ -581,7 +2742,7 @@
     <col min="8" max="8" width="10.83203125" customWidth="1"/>
     <col min="9" max="9" width="10.83203125" customWidth="1"/>
     <col min="10" max="10" width="10.83203125" customWidth="1"/>
-    <col min="11" max="11" width="10.83203125" customWidth="1"/>
+    <col min="11" max="11" width="13.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -621,12 +2782,77 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>No epics yet</v>
+        <v>Scikit-Learn/ API</v>
+      </c>
+      <c r="B2" t="str">
+        <v/>
+      </c>
+      <c r="C2" t="str">
+        <v>High</v>
+      </c>
+      <c r="D2">
+        <v>41</v>
+      </c>
+      <c r="E2">
+        <v>0</v>
+      </c>
+      <c r="F2">
+        <v>1</v>
+      </c>
+      <c r="G2">
+        <v>1</v>
+      </c>
+      <c r="H2">
+        <v>0</v>
+      </c>
+      <c r="I2">
+        <v>39</v>
+      </c>
+      <c r="J2" t="str">
+        <v>0%</v>
+      </c>
+      <c r="K2" t="str">
+        <v>Aug 8, 2026</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>Scikit-Learn/ User Guide</v>
+      </c>
+      <c r="B3" t="str">
+        <v/>
+      </c>
+      <c r="C3" t="str">
+        <v>High</v>
+      </c>
+      <c r="D3">
+        <v>15</v>
+      </c>
+      <c r="E3">
+        <v>0</v>
+      </c>
+      <c r="F3">
+        <v>0</v>
+      </c>
+      <c r="G3">
+        <v>0</v>
+      </c>
+      <c r="H3">
+        <v>0</v>
+      </c>
+      <c r="I3">
+        <v>15</v>
+      </c>
+      <c r="J3" t="str">
+        <v>0%</v>
+      </c>
+      <c r="K3" t="str">
+        <v>Aug 8, 2026</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:K2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:K3"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
feature : focus mode
</commit_message>
<xml_diff>
--- a/db/tracker.xlsx
+++ b/db/tracker.xlsx
@@ -412,8 +412,8 @@
     <col min="8" max="8" width="10.83203125" customWidth="1"/>
     <col min="9" max="9" width="10.83203125" customWidth="1"/>
     <col min="10" max="10" width="10.83203125" customWidth="1"/>
-    <col min="11" max="11" width="12.83203125" customWidth="1"/>
-    <col min="12" max="12" width="12.83203125" customWidth="1"/>
+    <col min="11" max="11" width="13.83203125" customWidth="1"/>
+    <col min="12" max="12" width="13.83203125" customWidth="1"/>
     <col min="13" max="13" width="15.83203125" customWidth="1"/>
   </cols>
   <sheetData>
@@ -490,10 +490,10 @@
         <v/>
       </c>
       <c r="K2" t="str">
-        <v>8 Aug 2026</v>
+        <v>Aug 8, 2026</v>
       </c>
       <c r="L2" t="str">
-        <v>8 Aug 2026</v>
+        <v>Aug 8, 2026</v>
       </c>
       <c r="M2" t="str">
         <v>mskjmm1ia28u3</v>
@@ -531,10 +531,10 @@
         <v/>
       </c>
       <c r="K3" t="str">
-        <v>8 Aug 2026</v>
+        <v>Aug 8, 2026</v>
       </c>
       <c r="L3" t="str">
-        <v>8 Aug 2026</v>
+        <v>Aug 8, 2026</v>
       </c>
       <c r="M3" t="str">
         <v>mskjmm1i9x9ut</v>
@@ -572,10 +572,10 @@
         <v/>
       </c>
       <c r="K4" t="str">
-        <v>8 Aug 2026</v>
+        <v>Aug 8, 2026</v>
       </c>
       <c r="L4" t="str">
-        <v>8 Aug 2026</v>
+        <v>Aug 8, 2026</v>
       </c>
       <c r="M4" t="str">
         <v>mskjmm1i0an4d</v>
@@ -613,10 +613,10 @@
         <v/>
       </c>
       <c r="K5" t="str">
-        <v>8 Aug 2026</v>
+        <v>Aug 8, 2026</v>
       </c>
       <c r="L5" t="str">
-        <v>8 Aug 2026</v>
+        <v>Aug 8, 2026</v>
       </c>
       <c r="M5" t="str">
         <v>mskjmm1ir8uys</v>
@@ -654,10 +654,10 @@
         <v/>
       </c>
       <c r="K6" t="str">
-        <v>8 Aug 2026</v>
+        <v>Aug 8, 2026</v>
       </c>
       <c r="L6" t="str">
-        <v>8 Aug 2026</v>
+        <v>Aug 8, 2026</v>
       </c>
       <c r="M6" t="str">
         <v>mskjmm1in1491</v>
@@ -695,10 +695,10 @@
         <v/>
       </c>
       <c r="K7" t="str">
-        <v>8 Aug 2026</v>
+        <v>Aug 8, 2026</v>
       </c>
       <c r="L7" t="str">
-        <v>8 Aug 2026</v>
+        <v>Aug 8, 2026</v>
       </c>
       <c r="M7" t="str">
         <v>mskjmm1iz5s6s</v>
@@ -736,10 +736,10 @@
         <v/>
       </c>
       <c r="K8" t="str">
-        <v>8 Aug 2026</v>
+        <v>Aug 8, 2026</v>
       </c>
       <c r="L8" t="str">
-        <v>8 Aug 2026</v>
+        <v>Aug 8, 2026</v>
       </c>
       <c r="M8" t="str">
         <v>mskjmm1iy83x2</v>
@@ -777,10 +777,10 @@
         <v/>
       </c>
       <c r="K9" t="str">
-        <v>8 Aug 2026</v>
+        <v>Aug 8, 2026</v>
       </c>
       <c r="L9" t="str">
-        <v>8 Aug 2026</v>
+        <v>Aug 8, 2026</v>
       </c>
       <c r="M9" t="str">
         <v>mskjmm1iahx06</v>
@@ -818,10 +818,10 @@
         <v/>
       </c>
       <c r="K10" t="str">
-        <v>8 Aug 2026</v>
+        <v>Aug 8, 2026</v>
       </c>
       <c r="L10" t="str">
-        <v>8 Aug 2026</v>
+        <v>Aug 8, 2026</v>
       </c>
       <c r="M10" t="str">
         <v>mskjmm1il6vzq</v>
@@ -859,10 +859,10 @@
         <v/>
       </c>
       <c r="K11" t="str">
-        <v>8 Aug 2026</v>
+        <v>Aug 8, 2026</v>
       </c>
       <c r="L11" t="str">
-        <v>8 Aug 2026</v>
+        <v>Aug 8, 2026</v>
       </c>
       <c r="M11" t="str">
         <v>mskjmm1idpwev</v>
@@ -900,10 +900,10 @@
         <v/>
       </c>
       <c r="K12" t="str">
-        <v>8 Aug 2026</v>
+        <v>Aug 8, 2026</v>
       </c>
       <c r="L12" t="str">
-        <v>8 Aug 2026</v>
+        <v>Aug 8, 2026</v>
       </c>
       <c r="M12" t="str">
         <v>mskjmm1irytor</v>
@@ -941,10 +941,10 @@
         <v/>
       </c>
       <c r="K13" t="str">
-        <v>8 Aug 2026</v>
+        <v>Aug 8, 2026</v>
       </c>
       <c r="L13" t="str">
-        <v>8 Aug 2026</v>
+        <v>Aug 8, 2026</v>
       </c>
       <c r="M13" t="str">
         <v>mskjmm1ijlwch</v>
@@ -982,10 +982,10 @@
         <v/>
       </c>
       <c r="K14" t="str">
-        <v>8 Aug 2026</v>
+        <v>Aug 8, 2026</v>
       </c>
       <c r="L14" t="str">
-        <v>8 Aug 2026</v>
+        <v>Aug 8, 2026</v>
       </c>
       <c r="M14" t="str">
         <v>mskjmm1izawzv</v>
@@ -1023,10 +1023,10 @@
         <v/>
       </c>
       <c r="K15" t="str">
-        <v>8 Aug 2026</v>
+        <v>Aug 8, 2026</v>
       </c>
       <c r="L15" t="str">
-        <v>8 Aug 2026</v>
+        <v>Aug 8, 2026</v>
       </c>
       <c r="M15" t="str">
         <v>mskjmm1i5vg3y</v>
@@ -1064,10 +1064,10 @@
         <v/>
       </c>
       <c r="K16" t="str">
-        <v>8 Aug 2026</v>
+        <v>Aug 8, 2026</v>
       </c>
       <c r="L16" t="str">
-        <v>8 Aug 2026</v>
+        <v>Aug 8, 2026</v>
       </c>
       <c r="M16" t="str">
         <v>mskjmm1ibeckq</v>
@@ -1105,10 +1105,10 @@
         <v/>
       </c>
       <c r="K17" t="str">
-        <v>8 Aug 2026</v>
+        <v>Aug 8, 2026</v>
       </c>
       <c r="L17" t="str">
-        <v>8 Aug 2026</v>
+        <v>Aug 8, 2026</v>
       </c>
       <c r="M17" t="str">
         <v>mskjuazrvir8z</v>
@@ -1146,10 +1146,10 @@
         <v/>
       </c>
       <c r="K18" t="str">
-        <v>8 Aug 2026</v>
+        <v>Aug 8, 2026</v>
       </c>
       <c r="L18" t="str">
-        <v>8 Aug 2026</v>
+        <v>Aug 8, 2026</v>
       </c>
       <c r="M18" t="str">
         <v>mskjuazrg15tu</v>
@@ -1187,10 +1187,10 @@
         <v/>
       </c>
       <c r="K19" t="str">
-        <v>8 Aug 2026</v>
+        <v>Aug 8, 2026</v>
       </c>
       <c r="L19" t="str">
-        <v>8 Aug 2026</v>
+        <v>Aug 8, 2026</v>
       </c>
       <c r="M19" t="str">
         <v>mskjuazrw6ksx</v>
@@ -1228,10 +1228,10 @@
         <v/>
       </c>
       <c r="K20" t="str">
-        <v>8 Aug 2026</v>
+        <v>Aug 8, 2026</v>
       </c>
       <c r="L20" t="str">
-        <v>8 Aug 2026</v>
+        <v>Aug 8, 2026</v>
       </c>
       <c r="M20" t="str">
         <v>mskjuazrdkxmj</v>
@@ -1269,10 +1269,10 @@
         <v/>
       </c>
       <c r="K21" t="str">
-        <v>8 Aug 2026</v>
+        <v>Aug 8, 2026</v>
       </c>
       <c r="L21" t="str">
-        <v>8 Aug 2026</v>
+        <v>Aug 8, 2026</v>
       </c>
       <c r="M21" t="str">
         <v>mskjuazrh7x1j</v>
@@ -1310,10 +1310,10 @@
         <v/>
       </c>
       <c r="K22" t="str">
-        <v>8 Aug 2026</v>
+        <v>Aug 8, 2026</v>
       </c>
       <c r="L22" t="str">
-        <v>8 Aug 2026</v>
+        <v>Aug 8, 2026</v>
       </c>
       <c r="M22" t="str">
         <v>mskjuazrqr7t0</v>
@@ -1351,10 +1351,10 @@
         <v/>
       </c>
       <c r="K23" t="str">
-        <v>8 Aug 2026</v>
+        <v>Aug 8, 2026</v>
       </c>
       <c r="L23" t="str">
-        <v>8 Aug 2026</v>
+        <v>Aug 8, 2026</v>
       </c>
       <c r="M23" t="str">
         <v>mskjuazruu4xz</v>
@@ -1392,10 +1392,10 @@
         <v/>
       </c>
       <c r="K24" t="str">
-        <v>8 Aug 2026</v>
+        <v>Aug 8, 2026</v>
       </c>
       <c r="L24" t="str">
-        <v>8 Aug 2026</v>
+        <v>Aug 8, 2026</v>
       </c>
       <c r="M24" t="str">
         <v>mskjuazr7izui</v>
@@ -1433,10 +1433,10 @@
         <v/>
       </c>
       <c r="K25" t="str">
-        <v>8 Aug 2026</v>
+        <v>Aug 8, 2026</v>
       </c>
       <c r="L25" t="str">
-        <v>8 Aug 2026</v>
+        <v>Aug 8, 2026</v>
       </c>
       <c r="M25" t="str">
         <v>mskjuazrk3kog</v>
@@ -1474,10 +1474,10 @@
         <v/>
       </c>
       <c r="K26" t="str">
-        <v>8 Aug 2026</v>
+        <v>Aug 8, 2026</v>
       </c>
       <c r="L26" t="str">
-        <v>8 Aug 2026</v>
+        <v>Aug 8, 2026</v>
       </c>
       <c r="M26" t="str">
         <v>mskjuazr76k5n</v>
@@ -1515,10 +1515,10 @@
         <v/>
       </c>
       <c r="K27" t="str">
-        <v>8 Aug 2026</v>
+        <v>Aug 8, 2026</v>
       </c>
       <c r="L27" t="str">
-        <v>8 Aug 2026</v>
+        <v>Aug 8, 2026</v>
       </c>
       <c r="M27" t="str">
         <v>mskjuazrr55s1</v>
@@ -1556,10 +1556,10 @@
         <v/>
       </c>
       <c r="K28" t="str">
-        <v>8 Aug 2026</v>
+        <v>Aug 8, 2026</v>
       </c>
       <c r="L28" t="str">
-        <v>8 Aug 2026</v>
+        <v>Aug 8, 2026</v>
       </c>
       <c r="M28" t="str">
         <v>mskjuazr0gaye</v>
@@ -1597,10 +1597,10 @@
         <v/>
       </c>
       <c r="K29" t="str">
-        <v>8 Aug 2026</v>
+        <v>Aug 8, 2026</v>
       </c>
       <c r="L29" t="str">
-        <v>8 Aug 2026</v>
+        <v>Aug 8, 2026</v>
       </c>
       <c r="M29" t="str">
         <v>mskjuazrqqxe7</v>
@@ -1638,10 +1638,10 @@
         <v/>
       </c>
       <c r="K30" t="str">
-        <v>8 Aug 2026</v>
+        <v>Aug 8, 2026</v>
       </c>
       <c r="L30" t="str">
-        <v>8 Aug 2026</v>
+        <v>Aug 8, 2026</v>
       </c>
       <c r="M30" t="str">
         <v>mskjuazrf8qko</v>
@@ -1679,10 +1679,10 @@
         <v/>
       </c>
       <c r="K31" t="str">
-        <v>8 Aug 2026</v>
+        <v>Aug 8, 2026</v>
       </c>
       <c r="L31" t="str">
-        <v>8 Aug 2026</v>
+        <v>Aug 8, 2026</v>
       </c>
       <c r="M31" t="str">
         <v>mskjuazrhf6l1</v>
@@ -1720,10 +1720,10 @@
         <v/>
       </c>
       <c r="K32" t="str">
-        <v>8 Aug 2026</v>
+        <v>Aug 8, 2026</v>
       </c>
       <c r="L32" t="str">
-        <v>8 Aug 2026</v>
+        <v>Aug 8, 2026</v>
       </c>
       <c r="M32" t="str">
         <v>mskjuazr6y2w1</v>
@@ -1761,10 +1761,10 @@
         <v/>
       </c>
       <c r="K33" t="str">
-        <v>8 Aug 2026</v>
+        <v>Aug 8, 2026</v>
       </c>
       <c r="L33" t="str">
-        <v>8 Aug 2026</v>
+        <v>Aug 8, 2026</v>
       </c>
       <c r="M33" t="str">
         <v>mskjuazr1qa1k</v>
@@ -1802,10 +1802,10 @@
         <v/>
       </c>
       <c r="K34" t="str">
-        <v>8 Aug 2026</v>
+        <v>Aug 8, 2026</v>
       </c>
       <c r="L34" t="str">
-        <v>8 Aug 2026</v>
+        <v>Aug 8, 2026</v>
       </c>
       <c r="M34" t="str">
         <v>mskjuazrjvhms</v>
@@ -1843,10 +1843,10 @@
         <v/>
       </c>
       <c r="K35" t="str">
-        <v>8 Aug 2026</v>
+        <v>Aug 8, 2026</v>
       </c>
       <c r="L35" t="str">
-        <v>8 Aug 2026</v>
+        <v>Aug 8, 2026</v>
       </c>
       <c r="M35" t="str">
         <v>mskjuazrxonbt</v>
@@ -1884,10 +1884,10 @@
         <v/>
       </c>
       <c r="K36" t="str">
-        <v>8 Aug 2026</v>
+        <v>Aug 8, 2026</v>
       </c>
       <c r="L36" t="str">
-        <v>8 Aug 2026</v>
+        <v>Aug 8, 2026</v>
       </c>
       <c r="M36" t="str">
         <v>mskjuazr4b0ct</v>
@@ -1925,10 +1925,10 @@
         <v/>
       </c>
       <c r="K37" t="str">
-        <v>8 Aug 2026</v>
+        <v>Aug 8, 2026</v>
       </c>
       <c r="L37" t="str">
-        <v>8 Aug 2026</v>
+        <v>Aug 8, 2026</v>
       </c>
       <c r="M37" t="str">
         <v>mskk12tpxnz6q</v>
@@ -2104,7 +2104,7 @@
     <col min="8" max="8" width="10.83203125" customWidth="1"/>
     <col min="9" max="9" width="10.83203125" customWidth="1"/>
     <col min="10" max="10" width="10.83203125" customWidth="1"/>
-    <col min="11" max="11" width="12.83203125" customWidth="1"/>
+    <col min="11" max="11" width="13.83203125" customWidth="1"/>
     <col min="12" max="12" width="15.83203125" customWidth="1"/>
   </cols>
   <sheetData>
@@ -2178,7 +2178,7 @@
         <v>0%</v>
       </c>
       <c r="K2" t="str">
-        <v>8 Aug 2026</v>
+        <v>Aug 8, 2026</v>
       </c>
       <c r="L2" t="str">
         <v>mskjl8cuwbnzs</v>
@@ -2216,7 +2216,7 @@
         <v>0%</v>
       </c>
       <c r="K3" t="str">
-        <v>8 Aug 2026</v>
+        <v>Aug 8, 2026</v>
       </c>
       <c r="L3" t="str">
         <v>mskjtuixm69sd</v>
@@ -2254,7 +2254,7 @@
         <v>0%</v>
       </c>
       <c r="K4" t="str">
-        <v>8 Aug 2026</v>
+        <v>Aug 8, 2026</v>
       </c>
       <c r="L4" t="str">
         <v>mskk074pigdwg</v>
@@ -2280,7 +2280,7 @@
     <col min="7" max="7" width="10.83203125" customWidth="1"/>
     <col min="8" max="8" width="10.83203125" customWidth="1"/>
     <col min="9" max="9" width="10.83203125" customWidth="1"/>
-    <col min="10" max="10" width="12.83203125" customWidth="1"/>
+    <col min="10" max="10" width="13.83203125" customWidth="1"/>
     <col min="11" max="11" width="15.83203125" customWidth="1"/>
   </cols>
   <sheetData>
@@ -2348,7 +2348,7 @@
         <v/>
       </c>
       <c r="J2" t="str">
-        <v>8 Aug 2026</v>
+        <v>Aug 8, 2026</v>
       </c>
       <c r="K2" t="str">
         <v>mskjvz8axp7bw</v>
@@ -2383,7 +2383,7 @@
         <v/>
       </c>
       <c r="J3" t="str">
-        <v>8 Aug 2026</v>
+        <v>Aug 8, 2026</v>
       </c>
       <c r="K3" t="str">
         <v>mskjw7zqqol4f</v>
@@ -2418,7 +2418,7 @@
         <v/>
       </c>
       <c r="J4" t="str">
-        <v>8 Aug 2026</v>
+        <v>Aug 8, 2026</v>
       </c>
       <c r="K4" t="str">
         <v>mskjwecwnzinb</v>
@@ -2453,7 +2453,7 @@
         <v/>
       </c>
       <c r="J5" t="str">
-        <v>8 Aug 2026</v>
+        <v>Aug 8, 2026</v>
       </c>
       <c r="K5" t="str">
         <v>mskjwjhp0kajz</v>
@@ -2488,7 +2488,7 @@
         <v/>
       </c>
       <c r="J6" t="str">
-        <v>8 Aug 2026</v>
+        <v>Aug 8, 2026</v>
       </c>
       <c r="K6" t="str">
         <v>mskjwo8nvlf63</v>
@@ -2523,7 +2523,7 @@
         <v/>
       </c>
       <c r="J7" t="str">
-        <v>8 Aug 2026</v>
+        <v>Aug 8, 2026</v>
       </c>
       <c r="K7" t="str">
         <v>mskjwtl16gyyh</v>
@@ -2566,7 +2566,7 @@
         <v/>
       </c>
       <c r="J8" t="str">
-        <v>8 Aug 2026</v>
+        <v>Aug 8, 2026</v>
       </c>
       <c r="K8" t="str">
         <v>mskk2136wm2x1</v>
@@ -2608,7 +2608,7 @@
         <v/>
       </c>
       <c r="J9" t="str">
-        <v>8 Aug 2026</v>
+        <v>Aug 8, 2026</v>
       </c>
       <c r="K9" t="str">
         <v>mskk2fgb7cnrq</v>
@@ -2659,7 +2659,7 @@
         <v/>
       </c>
       <c r="J10" t="str">
-        <v>8 Aug 2026</v>
+        <v>Aug 8, 2026</v>
       </c>
       <c r="K10" t="str">
         <v>mskk2w5rmle9n</v>

</xml_diff>

<commit_message>
fix : status udpate issue
</commit_message>
<xml_diff>
--- a/db/tracker.xlsx
+++ b/db/tracker.xlsx
@@ -412,8 +412,8 @@
     <col min="8" max="8" width="10.83203125" customWidth="1"/>
     <col min="9" max="9" width="10.83203125" customWidth="1"/>
     <col min="10" max="10" width="10.83203125" customWidth="1"/>
-    <col min="11" max="11" width="12.83203125" customWidth="1"/>
-    <col min="12" max="12" width="12.83203125" customWidth="1"/>
+    <col min="11" max="11" width="13.83203125" customWidth="1"/>
+    <col min="12" max="12" width="14.83203125" customWidth="1"/>
     <col min="13" max="13" width="15.83203125" customWidth="1"/>
   </cols>
   <sheetData>
@@ -478,7 +478,7 @@
         <v>2026-08</v>
       </c>
       <c r="G2" t="str">
-        <v>To Do</v>
+        <v>Done</v>
       </c>
       <c r="H2" t="str">
         <v>Low</v>
@@ -490,10 +490,10 @@
         <v/>
       </c>
       <c r="K2" t="str">
-        <v>8 Aug 2026</v>
+        <v>Aug 8, 2026</v>
       </c>
       <c r="L2" t="str">
-        <v>8 Aug 2026</v>
+        <v>Aug 10, 2026</v>
       </c>
       <c r="M2" t="str">
         <v>mskjmm1ia28u3</v>
@@ -519,7 +519,7 @@
         <v>2026-08</v>
       </c>
       <c r="G3" t="str">
-        <v>To Do</v>
+        <v>Done</v>
       </c>
       <c r="H3" t="str">
         <v>Low</v>
@@ -531,10 +531,10 @@
         <v/>
       </c>
       <c r="K3" t="str">
-        <v>8 Aug 2026</v>
+        <v>Aug 8, 2026</v>
       </c>
       <c r="L3" t="str">
-        <v>8 Aug 2026</v>
+        <v>Aug 10, 2026</v>
       </c>
       <c r="M3" t="str">
         <v>mskjmm1i9x9ut</v>
@@ -560,7 +560,7 @@
         <v>2026-08</v>
       </c>
       <c r="G4" t="str">
-        <v>To Do</v>
+        <v>Done</v>
       </c>
       <c r="H4" t="str">
         <v>Low</v>
@@ -572,10 +572,10 @@
         <v/>
       </c>
       <c r="K4" t="str">
-        <v>8 Aug 2026</v>
+        <v>Aug 8, 2026</v>
       </c>
       <c r="L4" t="str">
-        <v>8 Aug 2026</v>
+        <v>Aug 10, 2026</v>
       </c>
       <c r="M4" t="str">
         <v>mskjmm1i0an4d</v>
@@ -601,7 +601,7 @@
         <v>2026-08</v>
       </c>
       <c r="G5" t="str">
-        <v>To Do</v>
+        <v>Done</v>
       </c>
       <c r="H5" t="str">
         <v>Low</v>
@@ -613,10 +613,10 @@
         <v/>
       </c>
       <c r="K5" t="str">
-        <v>8 Aug 2026</v>
+        <v>Aug 8, 2026</v>
       </c>
       <c r="L5" t="str">
-        <v>8 Aug 2026</v>
+        <v>Aug 10, 2026</v>
       </c>
       <c r="M5" t="str">
         <v>mskjmm1ir8uys</v>
@@ -642,7 +642,7 @@
         <v>2026-08</v>
       </c>
       <c r="G6" t="str">
-        <v>To Do</v>
+        <v>Done</v>
       </c>
       <c r="H6" t="str">
         <v>Low</v>
@@ -654,10 +654,10 @@
         <v/>
       </c>
       <c r="K6" t="str">
-        <v>8 Aug 2026</v>
+        <v>Aug 8, 2026</v>
       </c>
       <c r="L6" t="str">
-        <v>8 Aug 2026</v>
+        <v>Aug 10, 2026</v>
       </c>
       <c r="M6" t="str">
         <v>mskjmm1in1491</v>
@@ -683,7 +683,7 @@
         <v>2026-08</v>
       </c>
       <c r="G7" t="str">
-        <v>To Do</v>
+        <v>Done</v>
       </c>
       <c r="H7" t="str">
         <v>Low</v>
@@ -695,10 +695,10 @@
         <v/>
       </c>
       <c r="K7" t="str">
-        <v>8 Aug 2026</v>
+        <v>Aug 8, 2026</v>
       </c>
       <c r="L7" t="str">
-        <v>8 Aug 2026</v>
+        <v>Aug 10, 2026</v>
       </c>
       <c r="M7" t="str">
         <v>mskjmm1iz5s6s</v>
@@ -724,7 +724,7 @@
         <v>2026-08</v>
       </c>
       <c r="G8" t="str">
-        <v>To Do</v>
+        <v>Done</v>
       </c>
       <c r="H8" t="str">
         <v>Low</v>
@@ -736,10 +736,10 @@
         <v/>
       </c>
       <c r="K8" t="str">
-        <v>8 Aug 2026</v>
+        <v>Aug 8, 2026</v>
       </c>
       <c r="L8" t="str">
-        <v>8 Aug 2026</v>
+        <v>Aug 10, 2026</v>
       </c>
       <c r="M8" t="str">
         <v>mskjmm1iy83x2</v>
@@ -777,10 +777,10 @@
         <v/>
       </c>
       <c r="K9" t="str">
-        <v>8 Aug 2026</v>
+        <v>Aug 8, 2026</v>
       </c>
       <c r="L9" t="str">
-        <v>8 Aug 2026</v>
+        <v>Aug 8, 2026</v>
       </c>
       <c r="M9" t="str">
         <v>mskjmm1iahx06</v>
@@ -818,10 +818,10 @@
         <v/>
       </c>
       <c r="K10" t="str">
-        <v>8 Aug 2026</v>
+        <v>Aug 8, 2026</v>
       </c>
       <c r="L10" t="str">
-        <v>8 Aug 2026</v>
+        <v>Aug 8, 2026</v>
       </c>
       <c r="M10" t="str">
         <v>mskjmm1il6vzq</v>
@@ -859,10 +859,10 @@
         <v/>
       </c>
       <c r="K11" t="str">
-        <v>8 Aug 2026</v>
+        <v>Aug 8, 2026</v>
       </c>
       <c r="L11" t="str">
-        <v>8 Aug 2026</v>
+        <v>Aug 8, 2026</v>
       </c>
       <c r="M11" t="str">
         <v>mskjmm1idpwev</v>
@@ -900,10 +900,10 @@
         <v/>
       </c>
       <c r="K12" t="str">
-        <v>8 Aug 2026</v>
+        <v>Aug 8, 2026</v>
       </c>
       <c r="L12" t="str">
-        <v>8 Aug 2026</v>
+        <v>Aug 8, 2026</v>
       </c>
       <c r="M12" t="str">
         <v>mskjmm1irytor</v>
@@ -941,10 +941,10 @@
         <v/>
       </c>
       <c r="K13" t="str">
-        <v>8 Aug 2026</v>
+        <v>Aug 8, 2026</v>
       </c>
       <c r="L13" t="str">
-        <v>8 Aug 2026</v>
+        <v>Aug 8, 2026</v>
       </c>
       <c r="M13" t="str">
         <v>mskjmm1ijlwch</v>
@@ -970,7 +970,7 @@
         <v>2026-08</v>
       </c>
       <c r="G14" t="str">
-        <v>To Do</v>
+        <v>Done</v>
       </c>
       <c r="H14" t="str">
         <v>Low</v>
@@ -982,10 +982,10 @@
         <v/>
       </c>
       <c r="K14" t="str">
-        <v>8 Aug 2026</v>
+        <v>Aug 8, 2026</v>
       </c>
       <c r="L14" t="str">
-        <v>8 Aug 2026</v>
+        <v>Aug 10, 2026</v>
       </c>
       <c r="M14" t="str">
         <v>mskjmm1izawzv</v>
@@ -1023,10 +1023,10 @@
         <v/>
       </c>
       <c r="K15" t="str">
-        <v>8 Aug 2026</v>
+        <v>Aug 8, 2026</v>
       </c>
       <c r="L15" t="str">
-        <v>8 Aug 2026</v>
+        <v>Aug 8, 2026</v>
       </c>
       <c r="M15" t="str">
         <v>mskjmm1i5vg3y</v>
@@ -1064,10 +1064,10 @@
         <v/>
       </c>
       <c r="K16" t="str">
-        <v>8 Aug 2026</v>
+        <v>Aug 8, 2026</v>
       </c>
       <c r="L16" t="str">
-        <v>8 Aug 2026</v>
+        <v>Aug 8, 2026</v>
       </c>
       <c r="M16" t="str">
         <v>mskjmm1ibeckq</v>
@@ -1105,10 +1105,10 @@
         <v/>
       </c>
       <c r="K17" t="str">
-        <v>8 Aug 2026</v>
+        <v>Aug 8, 2026</v>
       </c>
       <c r="L17" t="str">
-        <v>8 Aug 2026</v>
+        <v>Aug 8, 2026</v>
       </c>
       <c r="M17" t="str">
         <v>mskjuazrvir8z</v>
@@ -1146,10 +1146,10 @@
         <v/>
       </c>
       <c r="K18" t="str">
-        <v>8 Aug 2026</v>
+        <v>Aug 8, 2026</v>
       </c>
       <c r="L18" t="str">
-        <v>8 Aug 2026</v>
+        <v>Aug 8, 2026</v>
       </c>
       <c r="M18" t="str">
         <v>mskjuazrg15tu</v>
@@ -1187,10 +1187,10 @@
         <v/>
       </c>
       <c r="K19" t="str">
-        <v>8 Aug 2026</v>
+        <v>Aug 8, 2026</v>
       </c>
       <c r="L19" t="str">
-        <v>8 Aug 2026</v>
+        <v>Aug 8, 2026</v>
       </c>
       <c r="M19" t="str">
         <v>mskjuazrw6ksx</v>
@@ -1228,10 +1228,10 @@
         <v/>
       </c>
       <c r="K20" t="str">
-        <v>8 Aug 2026</v>
+        <v>Aug 8, 2026</v>
       </c>
       <c r="L20" t="str">
-        <v>8 Aug 2026</v>
+        <v>Aug 8, 2026</v>
       </c>
       <c r="M20" t="str">
         <v>mskjuazrdkxmj</v>
@@ -1269,10 +1269,10 @@
         <v/>
       </c>
       <c r="K21" t="str">
-        <v>8 Aug 2026</v>
+        <v>Aug 8, 2026</v>
       </c>
       <c r="L21" t="str">
-        <v>8 Aug 2026</v>
+        <v>Aug 8, 2026</v>
       </c>
       <c r="M21" t="str">
         <v>mskjuazrh7x1j</v>
@@ -1310,10 +1310,10 @@
         <v/>
       </c>
       <c r="K22" t="str">
-        <v>8 Aug 2026</v>
+        <v>Aug 8, 2026</v>
       </c>
       <c r="L22" t="str">
-        <v>8 Aug 2026</v>
+        <v>Aug 8, 2026</v>
       </c>
       <c r="M22" t="str">
         <v>mskjuazrqr7t0</v>
@@ -1351,10 +1351,10 @@
         <v/>
       </c>
       <c r="K23" t="str">
-        <v>8 Aug 2026</v>
+        <v>Aug 8, 2026</v>
       </c>
       <c r="L23" t="str">
-        <v>8 Aug 2026</v>
+        <v>Aug 8, 2026</v>
       </c>
       <c r="M23" t="str">
         <v>mskjuazruu4xz</v>
@@ -1392,10 +1392,10 @@
         <v/>
       </c>
       <c r="K24" t="str">
-        <v>8 Aug 2026</v>
+        <v>Aug 8, 2026</v>
       </c>
       <c r="L24" t="str">
-        <v>8 Aug 2026</v>
+        <v>Aug 8, 2026</v>
       </c>
       <c r="M24" t="str">
         <v>mskjuazr7izui</v>
@@ -1433,10 +1433,10 @@
         <v/>
       </c>
       <c r="K25" t="str">
-        <v>8 Aug 2026</v>
+        <v>Aug 8, 2026</v>
       </c>
       <c r="L25" t="str">
-        <v>8 Aug 2026</v>
+        <v>Aug 8, 2026</v>
       </c>
       <c r="M25" t="str">
         <v>mskjuazrk3kog</v>
@@ -1474,10 +1474,10 @@
         <v/>
       </c>
       <c r="K26" t="str">
-        <v>8 Aug 2026</v>
+        <v>Aug 8, 2026</v>
       </c>
       <c r="L26" t="str">
-        <v>8 Aug 2026</v>
+        <v>Aug 8, 2026</v>
       </c>
       <c r="M26" t="str">
         <v>mskjuazr76k5n</v>
@@ -1515,10 +1515,10 @@
         <v/>
       </c>
       <c r="K27" t="str">
-        <v>8 Aug 2026</v>
+        <v>Aug 8, 2026</v>
       </c>
       <c r="L27" t="str">
-        <v>8 Aug 2026</v>
+        <v>Aug 8, 2026</v>
       </c>
       <c r="M27" t="str">
         <v>mskjuazrr55s1</v>
@@ -1556,10 +1556,10 @@
         <v/>
       </c>
       <c r="K28" t="str">
-        <v>8 Aug 2026</v>
+        <v>Aug 8, 2026</v>
       </c>
       <c r="L28" t="str">
-        <v>8 Aug 2026</v>
+        <v>Aug 8, 2026</v>
       </c>
       <c r="M28" t="str">
         <v>mskjuazr0gaye</v>
@@ -1597,10 +1597,10 @@
         <v/>
       </c>
       <c r="K29" t="str">
-        <v>8 Aug 2026</v>
+        <v>Aug 8, 2026</v>
       </c>
       <c r="L29" t="str">
-        <v>8 Aug 2026</v>
+        <v>Aug 8, 2026</v>
       </c>
       <c r="M29" t="str">
         <v>mskjuazrqqxe7</v>
@@ -1638,10 +1638,10 @@
         <v/>
       </c>
       <c r="K30" t="str">
-        <v>8 Aug 2026</v>
+        <v>Aug 8, 2026</v>
       </c>
       <c r="L30" t="str">
-        <v>8 Aug 2026</v>
+        <v>Aug 8, 2026</v>
       </c>
       <c r="M30" t="str">
         <v>mskjuazrf8qko</v>
@@ -1679,10 +1679,10 @@
         <v/>
       </c>
       <c r="K31" t="str">
-        <v>8 Aug 2026</v>
+        <v>Aug 8, 2026</v>
       </c>
       <c r="L31" t="str">
-        <v>8 Aug 2026</v>
+        <v>Aug 8, 2026</v>
       </c>
       <c r="M31" t="str">
         <v>mskjuazrhf6l1</v>
@@ -1720,10 +1720,10 @@
         <v/>
       </c>
       <c r="K32" t="str">
-        <v>8 Aug 2026</v>
+        <v>Aug 8, 2026</v>
       </c>
       <c r="L32" t="str">
-        <v>8 Aug 2026</v>
+        <v>Aug 8, 2026</v>
       </c>
       <c r="M32" t="str">
         <v>mskjuazr6y2w1</v>
@@ -1761,10 +1761,10 @@
         <v/>
       </c>
       <c r="K33" t="str">
-        <v>8 Aug 2026</v>
+        <v>Aug 8, 2026</v>
       </c>
       <c r="L33" t="str">
-        <v>8 Aug 2026</v>
+        <v>Aug 8, 2026</v>
       </c>
       <c r="M33" t="str">
         <v>mskjuazr1qa1k</v>
@@ -1802,10 +1802,10 @@
         <v/>
       </c>
       <c r="K34" t="str">
-        <v>8 Aug 2026</v>
+        <v>Aug 8, 2026</v>
       </c>
       <c r="L34" t="str">
-        <v>8 Aug 2026</v>
+        <v>Aug 8, 2026</v>
       </c>
       <c r="M34" t="str">
         <v>mskjuazrjvhms</v>
@@ -1843,10 +1843,10 @@
         <v/>
       </c>
       <c r="K35" t="str">
-        <v>8 Aug 2026</v>
+        <v>Aug 8, 2026</v>
       </c>
       <c r="L35" t="str">
-        <v>8 Aug 2026</v>
+        <v>Aug 8, 2026</v>
       </c>
       <c r="M35" t="str">
         <v>mskjuazrxonbt</v>
@@ -1884,10 +1884,10 @@
         <v/>
       </c>
       <c r="K36" t="str">
-        <v>8 Aug 2026</v>
+        <v>Aug 8, 2026</v>
       </c>
       <c r="L36" t="str">
-        <v>8 Aug 2026</v>
+        <v>Aug 8, 2026</v>
       </c>
       <c r="M36" t="str">
         <v>mskjuazr4b0ct</v>
@@ -1925,10 +1925,10 @@
         <v/>
       </c>
       <c r="K37" t="str">
-        <v>8 Aug 2026</v>
+        <v>Aug 8, 2026</v>
       </c>
       <c r="L37" t="str">
-        <v>8 Aug 2026</v>
+        <v>Aug 8, 2026</v>
       </c>
       <c r="M37" t="str">
         <v>mskk12tpxnz6q</v>
@@ -2062,7 +2062,7 @@
         <v>18</v>
       </c>
       <c r="G3">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="H3">
         <v>0</v>
@@ -2074,10 +2074,10 @@
         <v>0</v>
       </c>
       <c r="K3">
-        <v>18</v>
+        <v>10</v>
       </c>
       <c r="L3" t="str">
-        <v>0%</v>
+        <v>44%</v>
       </c>
       <c r="M3" t="str">
         <v>mskjojd2g5ua7</v>
@@ -2104,7 +2104,7 @@
     <col min="8" max="8" width="10.83203125" customWidth="1"/>
     <col min="9" max="9" width="10.83203125" customWidth="1"/>
     <col min="10" max="10" width="10.83203125" customWidth="1"/>
-    <col min="11" max="11" width="12.83203125" customWidth="1"/>
+    <col min="11" max="11" width="13.83203125" customWidth="1"/>
     <col min="12" max="12" width="18.83203125" customWidth="1"/>
     <col min="13" max="13" width="16.83203125" customWidth="1"/>
     <col min="14" max="14" width="16.83203125" customWidth="1"/>
@@ -2180,7 +2180,7 @@
         <v>15</v>
       </c>
       <c r="E2">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="F2">
         <v>0</v>
@@ -2192,13 +2192,13 @@
         <v>0</v>
       </c>
       <c r="I2">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="J2" t="str">
-        <v>0%</v>
+        <v>53%</v>
       </c>
       <c r="K2" t="str">
-        <v>8 Aug 2026</v>
+        <v>Aug 8, 2026</v>
       </c>
       <c r="L2" t="str">
         <v>FALSE</v>
@@ -2251,7 +2251,7 @@
         <v>0%</v>
       </c>
       <c r="K3" t="str">
-        <v>8 Aug 2026</v>
+        <v>Aug 8, 2026</v>
       </c>
       <c r="L3" t="str">
         <v>FALSE</v>
@@ -2304,7 +2304,7 @@
         <v>0%</v>
       </c>
       <c r="K4" t="str">
-        <v>8 Aug 2026</v>
+        <v>Aug 8, 2026</v>
       </c>
       <c r="L4" t="str">
         <v>FALSE</v>
@@ -2345,7 +2345,7 @@
     <col min="7" max="7" width="10.83203125" customWidth="1"/>
     <col min="8" max="8" width="10.83203125" customWidth="1"/>
     <col min="9" max="9" width="10.83203125" customWidth="1"/>
-    <col min="10" max="10" width="12.83203125" customWidth="1"/>
+    <col min="10" max="10" width="13.83203125" customWidth="1"/>
     <col min="11" max="11" width="15.83203125" customWidth="1"/>
   </cols>
   <sheetData>
@@ -2413,7 +2413,7 @@
         <v/>
       </c>
       <c r="J2" t="str">
-        <v>8 Aug 2026</v>
+        <v>Aug 8, 2026</v>
       </c>
       <c r="K2" t="str">
         <v>mskjvz8axp7bw</v>
@@ -2448,7 +2448,7 @@
         <v/>
       </c>
       <c r="J3" t="str">
-        <v>8 Aug 2026</v>
+        <v>Aug 8, 2026</v>
       </c>
       <c r="K3" t="str">
         <v>mskjw7zqqol4f</v>
@@ -2483,7 +2483,7 @@
         <v/>
       </c>
       <c r="J4" t="str">
-        <v>8 Aug 2026</v>
+        <v>Aug 8, 2026</v>
       </c>
       <c r="K4" t="str">
         <v>mskjwecwnzinb</v>
@@ -2518,7 +2518,7 @@
         <v/>
       </c>
       <c r="J5" t="str">
-        <v>8 Aug 2026</v>
+        <v>Aug 8, 2026</v>
       </c>
       <c r="K5" t="str">
         <v>mskjwjhp0kajz</v>
@@ -2553,7 +2553,7 @@
         <v/>
       </c>
       <c r="J6" t="str">
-        <v>8 Aug 2026</v>
+        <v>Aug 8, 2026</v>
       </c>
       <c r="K6" t="str">
         <v>mskjwo8nvlf63</v>
@@ -2588,7 +2588,7 @@
         <v/>
       </c>
       <c r="J7" t="str">
-        <v>8 Aug 2026</v>
+        <v>Aug 8, 2026</v>
       </c>
       <c r="K7" t="str">
         <v>mskjwtl16gyyh</v>
@@ -2631,7 +2631,7 @@
         <v/>
       </c>
       <c r="J8" t="str">
-        <v>8 Aug 2026</v>
+        <v>Aug 8, 2026</v>
       </c>
       <c r="K8" t="str">
         <v>mskk2136wm2x1</v>
@@ -2673,7 +2673,7 @@
         <v/>
       </c>
       <c r="J9" t="str">
-        <v>8 Aug 2026</v>
+        <v>Aug 8, 2026</v>
       </c>
       <c r="K9" t="str">
         <v>mskk2fgb7cnrq</v>
@@ -2724,7 +2724,7 @@
         <v/>
       </c>
       <c r="J10" t="str">
-        <v>8 Aug 2026</v>
+        <v>Aug 8, 2026</v>
       </c>
       <c r="K10" t="str">
         <v>mskk2w5rmle9n</v>

</xml_diff>

<commit_message>
fix: schuled task issues
</commit_message>
<xml_diff>
--- a/db/tracker.xlsx
+++ b/db/tracker.xlsx
@@ -412,8 +412,8 @@
     <col min="8" max="8" width="10.83203125" customWidth="1"/>
     <col min="9" max="9" width="10.83203125" customWidth="1"/>
     <col min="10" max="10" width="10.83203125" customWidth="1"/>
-    <col min="11" max="11" width="13.83203125" customWidth="1"/>
-    <col min="12" max="12" width="13.83203125" customWidth="1"/>
+    <col min="11" max="11" width="14.83203125" customWidth="1"/>
+    <col min="12" max="12" width="14.83203125" customWidth="1"/>
     <col min="13" max="13" width="15.83203125" customWidth="1"/>
   </cols>
   <sheetData>
@@ -490,10 +490,10 @@
         <v/>
       </c>
       <c r="K2" t="str">
-        <v>8 Aug 2026</v>
+        <v>Aug 8, 2026</v>
       </c>
       <c r="L2" t="str">
-        <v>10 Aug 2026</v>
+        <v>Aug 10, 2026</v>
       </c>
       <c r="M2" t="str">
         <v>mskjmm1ia28u3</v>
@@ -531,10 +531,10 @@
         <v/>
       </c>
       <c r="K3" t="str">
-        <v>8 Aug 2026</v>
+        <v>Aug 8, 2026</v>
       </c>
       <c r="L3" t="str">
-        <v>10 Aug 2026</v>
+        <v>Aug 10, 2026</v>
       </c>
       <c r="M3" t="str">
         <v>mskjmm1i9x9ut</v>
@@ -572,10 +572,10 @@
         <v/>
       </c>
       <c r="K4" t="str">
-        <v>8 Aug 2026</v>
+        <v>Aug 8, 2026</v>
       </c>
       <c r="L4" t="str">
-        <v>10 Aug 2026</v>
+        <v>Aug 10, 2026</v>
       </c>
       <c r="M4" t="str">
         <v>mskjmm1i0an4d</v>
@@ -613,10 +613,10 @@
         <v/>
       </c>
       <c r="K5" t="str">
-        <v>8 Aug 2026</v>
+        <v>Aug 8, 2026</v>
       </c>
       <c r="L5" t="str">
-        <v>10 Aug 2026</v>
+        <v>Aug 10, 2026</v>
       </c>
       <c r="M5" t="str">
         <v>mskjmm1ir8uys</v>
@@ -654,10 +654,10 @@
         <v/>
       </c>
       <c r="K6" t="str">
-        <v>8 Aug 2026</v>
+        <v>Aug 8, 2026</v>
       </c>
       <c r="L6" t="str">
-        <v>10 Aug 2026</v>
+        <v>Aug 10, 2026</v>
       </c>
       <c r="M6" t="str">
         <v>mskjmm1in1491</v>
@@ -695,10 +695,10 @@
         <v/>
       </c>
       <c r="K7" t="str">
-        <v>8 Aug 2026</v>
+        <v>Aug 8, 2026</v>
       </c>
       <c r="L7" t="str">
-        <v>10 Aug 2026</v>
+        <v>Aug 10, 2026</v>
       </c>
       <c r="M7" t="str">
         <v>mskjmm1iz5s6s</v>
@@ -736,10 +736,10 @@
         <v/>
       </c>
       <c r="K8" t="str">
-        <v>8 Aug 2026</v>
+        <v>Aug 8, 2026</v>
       </c>
       <c r="L8" t="str">
-        <v>10 Aug 2026</v>
+        <v>Aug 10, 2026</v>
       </c>
       <c r="M8" t="str">
         <v>mskjmm1iy83x2</v>
@@ -777,10 +777,10 @@
         <v/>
       </c>
       <c r="K9" t="str">
-        <v>8 Aug 2026</v>
+        <v>Aug 8, 2026</v>
       </c>
       <c r="L9" t="str">
-        <v>8 Aug 2026</v>
+        <v>Aug 8, 2026</v>
       </c>
       <c r="M9" t="str">
         <v>mskjmm1iahx06</v>
@@ -818,10 +818,10 @@
         <v/>
       </c>
       <c r="K10" t="str">
-        <v>8 Aug 2026</v>
+        <v>Aug 8, 2026</v>
       </c>
       <c r="L10" t="str">
-        <v>8 Aug 2026</v>
+        <v>Aug 8, 2026</v>
       </c>
       <c r="M10" t="str">
         <v>mskjmm1il6vzq</v>
@@ -859,10 +859,10 @@
         <v/>
       </c>
       <c r="K11" t="str">
-        <v>8 Aug 2026</v>
+        <v>Aug 8, 2026</v>
       </c>
       <c r="L11" t="str">
-        <v>8 Aug 2026</v>
+        <v>Aug 8, 2026</v>
       </c>
       <c r="M11" t="str">
         <v>mskjmm1idpwev</v>
@@ -900,10 +900,10 @@
         <v/>
       </c>
       <c r="K12" t="str">
-        <v>8 Aug 2026</v>
+        <v>Aug 8, 2026</v>
       </c>
       <c r="L12" t="str">
-        <v>8 Aug 2026</v>
+        <v>Aug 8, 2026</v>
       </c>
       <c r="M12" t="str">
         <v>mskjmm1irytor</v>
@@ -941,10 +941,10 @@
         <v/>
       </c>
       <c r="K13" t="str">
-        <v>8 Aug 2026</v>
+        <v>Aug 8, 2026</v>
       </c>
       <c r="L13" t="str">
-        <v>8 Aug 2026</v>
+        <v>Aug 8, 2026</v>
       </c>
       <c r="M13" t="str">
         <v>mskjmm1ijlwch</v>
@@ -982,10 +982,10 @@
         <v/>
       </c>
       <c r="K14" t="str">
-        <v>8 Aug 2026</v>
+        <v>Aug 8, 2026</v>
       </c>
       <c r="L14" t="str">
-        <v>10 Aug 2026</v>
+        <v>Aug 10, 2026</v>
       </c>
       <c r="M14" t="str">
         <v>mskjmm1izawzv</v>
@@ -1023,10 +1023,10 @@
         <v/>
       </c>
       <c r="K15" t="str">
-        <v>8 Aug 2026</v>
+        <v>Aug 8, 2026</v>
       </c>
       <c r="L15" t="str">
-        <v>8 Aug 2026</v>
+        <v>Aug 8, 2026</v>
       </c>
       <c r="M15" t="str">
         <v>mskjmm1i5vg3y</v>
@@ -1064,10 +1064,10 @@
         <v/>
       </c>
       <c r="K16" t="str">
-        <v>8 Aug 2026</v>
+        <v>Aug 8, 2026</v>
       </c>
       <c r="L16" t="str">
-        <v>8 Aug 2026</v>
+        <v>Aug 8, 2026</v>
       </c>
       <c r="M16" t="str">
         <v>mskjmm1ibeckq</v>
@@ -1105,10 +1105,10 @@
         <v/>
       </c>
       <c r="K17" t="str">
-        <v>8 Aug 2026</v>
+        <v>Aug 8, 2026</v>
       </c>
       <c r="L17" t="str">
-        <v>10 Aug 2026</v>
+        <v>Aug 10, 2026</v>
       </c>
       <c r="M17" t="str">
         <v>mskjuazrvir8z</v>
@@ -1146,10 +1146,10 @@
         <v/>
       </c>
       <c r="K18" t="str">
-        <v>8 Aug 2026</v>
+        <v>Aug 8, 2026</v>
       </c>
       <c r="L18" t="str">
-        <v>10 Aug 2026</v>
+        <v>Aug 10, 2026</v>
       </c>
       <c r="M18" t="str">
         <v>mskjuazrg15tu</v>
@@ -1187,10 +1187,10 @@
         <v/>
       </c>
       <c r="K19" t="str">
-        <v>8 Aug 2026</v>
+        <v>Aug 8, 2026</v>
       </c>
       <c r="L19" t="str">
-        <v>10 Aug 2026</v>
+        <v>Aug 10, 2026</v>
       </c>
       <c r="M19" t="str">
         <v>mskjuazrw6ksx</v>
@@ -1228,10 +1228,10 @@
         <v/>
       </c>
       <c r="K20" t="str">
-        <v>8 Aug 2026</v>
+        <v>Aug 8, 2026</v>
       </c>
       <c r="L20" t="str">
-        <v>10 Aug 2026</v>
+        <v>Aug 10, 2026</v>
       </c>
       <c r="M20" t="str">
         <v>mskjuazrdkxmj</v>
@@ -1269,10 +1269,10 @@
         <v/>
       </c>
       <c r="K21" t="str">
-        <v>8 Aug 2026</v>
+        <v>Aug 8, 2026</v>
       </c>
       <c r="L21" t="str">
-        <v>8 Aug 2026</v>
+        <v>Aug 8, 2026</v>
       </c>
       <c r="M21" t="str">
         <v>mskjuazrh7x1j</v>
@@ -1310,10 +1310,10 @@
         <v/>
       </c>
       <c r="K22" t="str">
-        <v>8 Aug 2026</v>
+        <v>Aug 8, 2026</v>
       </c>
       <c r="L22" t="str">
-        <v>8 Aug 2026</v>
+        <v>Aug 8, 2026</v>
       </c>
       <c r="M22" t="str">
         <v>mskjuazrqr7t0</v>
@@ -1351,10 +1351,10 @@
         <v/>
       </c>
       <c r="K23" t="str">
-        <v>8 Aug 2026</v>
+        <v>Aug 8, 2026</v>
       </c>
       <c r="L23" t="str">
-        <v>10 Aug 2026</v>
+        <v>Aug 10, 2026</v>
       </c>
       <c r="M23" t="str">
         <v>mskjuazruu4xz</v>
@@ -1392,10 +1392,10 @@
         <v/>
       </c>
       <c r="K24" t="str">
-        <v>8 Aug 2026</v>
+        <v>Aug 8, 2026</v>
       </c>
       <c r="L24" t="str">
-        <v>10 Aug 2026</v>
+        <v>Aug 10, 2026</v>
       </c>
       <c r="M24" t="str">
         <v>mskjuazr7izui</v>
@@ -1433,10 +1433,10 @@
         <v/>
       </c>
       <c r="K25" t="str">
-        <v>8 Aug 2026</v>
+        <v>Aug 8, 2026</v>
       </c>
       <c r="L25" t="str">
-        <v>10 Aug 2026</v>
+        <v>Aug 10, 2026</v>
       </c>
       <c r="M25" t="str">
         <v>mskjuazrk3kog</v>
@@ -1474,10 +1474,10 @@
         <v/>
       </c>
       <c r="K26" t="str">
-        <v>8 Aug 2026</v>
+        <v>Aug 8, 2026</v>
       </c>
       <c r="L26" t="str">
-        <v>8 Aug 2026</v>
+        <v>Aug 8, 2026</v>
       </c>
       <c r="M26" t="str">
         <v>mskjuazr76k5n</v>
@@ -1515,10 +1515,10 @@
         <v/>
       </c>
       <c r="K27" t="str">
-        <v>8 Aug 2026</v>
+        <v>Aug 8, 2026</v>
       </c>
       <c r="L27" t="str">
-        <v>8 Aug 2026</v>
+        <v>Aug 8, 2026</v>
       </c>
       <c r="M27" t="str">
         <v>mskjuazrr55s1</v>
@@ -1556,10 +1556,10 @@
         <v/>
       </c>
       <c r="K28" t="str">
-        <v>8 Aug 2026</v>
+        <v>Aug 8, 2026</v>
       </c>
       <c r="L28" t="str">
-        <v>8 Aug 2026</v>
+        <v>Aug 8, 2026</v>
       </c>
       <c r="M28" t="str">
         <v>mskjuazr0gaye</v>
@@ -1597,10 +1597,10 @@
         <v/>
       </c>
       <c r="K29" t="str">
-        <v>8 Aug 2026</v>
+        <v>Aug 8, 2026</v>
       </c>
       <c r="L29" t="str">
-        <v>8 Aug 2026</v>
+        <v>Aug 8, 2026</v>
       </c>
       <c r="M29" t="str">
         <v>mskjuazrqqxe7</v>
@@ -1638,10 +1638,10 @@
         <v/>
       </c>
       <c r="K30" t="str">
-        <v>8 Aug 2026</v>
+        <v>Aug 8, 2026</v>
       </c>
       <c r="L30" t="str">
-        <v>8 Aug 2026</v>
+        <v>Aug 8, 2026</v>
       </c>
       <c r="M30" t="str">
         <v>mskjuazrf8qko</v>
@@ -1679,10 +1679,10 @@
         <v/>
       </c>
       <c r="K31" t="str">
-        <v>8 Aug 2026</v>
+        <v>Aug 8, 2026</v>
       </c>
       <c r="L31" t="str">
-        <v>8 Aug 2026</v>
+        <v>Aug 8, 2026</v>
       </c>
       <c r="M31" t="str">
         <v>mskjuazrhf6l1</v>
@@ -1720,10 +1720,10 @@
         <v/>
       </c>
       <c r="K32" t="str">
-        <v>8 Aug 2026</v>
+        <v>Aug 8, 2026</v>
       </c>
       <c r="L32" t="str">
-        <v>8 Aug 2026</v>
+        <v>Aug 8, 2026</v>
       </c>
       <c r="M32" t="str">
         <v>mskjuazr6y2w1</v>
@@ -1761,10 +1761,10 @@
         <v/>
       </c>
       <c r="K33" t="str">
-        <v>8 Aug 2026</v>
+        <v>Aug 8, 2026</v>
       </c>
       <c r="L33" t="str">
-        <v>8 Aug 2026</v>
+        <v>Aug 8, 2026</v>
       </c>
       <c r="M33" t="str">
         <v>mskjuazr1qa1k</v>
@@ -1802,10 +1802,10 @@
         <v/>
       </c>
       <c r="K34" t="str">
-        <v>8 Aug 2026</v>
+        <v>Aug 8, 2026</v>
       </c>
       <c r="L34" t="str">
-        <v>8 Aug 2026</v>
+        <v>Aug 8, 2026</v>
       </c>
       <c r="M34" t="str">
         <v>mskjuazrjvhms</v>
@@ -1843,10 +1843,10 @@
         <v/>
       </c>
       <c r="K35" t="str">
-        <v>8 Aug 2026</v>
+        <v>Aug 8, 2026</v>
       </c>
       <c r="L35" t="str">
-        <v>8 Aug 2026</v>
+        <v>Aug 8, 2026</v>
       </c>
       <c r="M35" t="str">
         <v>mskjuazrxonbt</v>
@@ -1884,10 +1884,10 @@
         <v/>
       </c>
       <c r="K36" t="str">
-        <v>8 Aug 2026</v>
+        <v>Aug 8, 2026</v>
       </c>
       <c r="L36" t="str">
-        <v>8 Aug 2026</v>
+        <v>Aug 8, 2026</v>
       </c>
       <c r="M36" t="str">
         <v>mskjuazr4b0ct</v>
@@ -1925,10 +1925,10 @@
         <v/>
       </c>
       <c r="K37" t="str">
-        <v>8 Aug 2026</v>
+        <v>Aug 8, 2026</v>
       </c>
       <c r="L37" t="str">
-        <v>11 Aug 2026</v>
+        <v>Aug 11, 2026</v>
       </c>
       <c r="M37" t="str">
         <v>mskk12tpxnz6q</v>
@@ -1966,10 +1966,10 @@
         <v/>
       </c>
       <c r="K38" t="str">
-        <v>11 Aug 2026</v>
+        <v>Aug 11, 2026</v>
       </c>
       <c r="L38" t="str">
-        <v>11 Aug 2026</v>
+        <v>Aug 11, 2026</v>
       </c>
       <c r="M38" t="str">
         <v>msokvqo38bfww</v>
@@ -2007,10 +2007,10 @@
         <v/>
       </c>
       <c r="K39" t="str">
-        <v>11 Aug 2026</v>
+        <v>Aug 11, 2026</v>
       </c>
       <c r="L39" t="str">
-        <v>11 Aug 2026</v>
+        <v>Aug 11, 2026</v>
       </c>
       <c r="M39" t="str">
         <v>msokvqo3tpfld</v>
@@ -2048,10 +2048,10 @@
         <v/>
       </c>
       <c r="K40" t="str">
-        <v>11 Aug 2026</v>
+        <v>Aug 11, 2026</v>
       </c>
       <c r="L40" t="str">
-        <v>11 Aug 2026</v>
+        <v>Aug 11, 2026</v>
       </c>
       <c r="M40" t="str">
         <v>msokvqo323mt3</v>
@@ -2089,10 +2089,10 @@
         <v/>
       </c>
       <c r="K41" t="str">
-        <v>11 Aug 2026</v>
+        <v>Aug 11, 2026</v>
       </c>
       <c r="L41" t="str">
-        <v>11 Aug 2026</v>
+        <v>Aug 11, 2026</v>
       </c>
       <c r="M41" t="str">
         <v>msokvqo3fjm2f</v>
@@ -2130,10 +2130,10 @@
         <v/>
       </c>
       <c r="K42" t="str">
-        <v>11 Aug 2026</v>
+        <v>Aug 11, 2026</v>
       </c>
       <c r="L42" t="str">
-        <v>11 Aug 2026</v>
+        <v>Aug 11, 2026</v>
       </c>
       <c r="M42" t="str">
         <v>msokvqo34hlxf</v>
@@ -2171,10 +2171,10 @@
         <v/>
       </c>
       <c r="K43" t="str">
-        <v>11 Aug 2026</v>
+        <v>Aug 11, 2026</v>
       </c>
       <c r="L43" t="str">
-        <v>11 Aug 2026</v>
+        <v>Aug 11, 2026</v>
       </c>
       <c r="M43" t="str">
         <v>msokwhmdho1q0</v>
@@ -2212,10 +2212,10 @@
         <v/>
       </c>
       <c r="K44" t="str">
-        <v>11 Aug 2026</v>
+        <v>Aug 11, 2026</v>
       </c>
       <c r="L44" t="str">
-        <v>11 Aug 2026</v>
+        <v>Aug 11, 2026</v>
       </c>
       <c r="M44" t="str">
         <v>msokwhmdegi75</v>
@@ -2253,10 +2253,10 @@
         <v/>
       </c>
       <c r="K45" t="str">
-        <v>11 Aug 2026</v>
+        <v>Aug 11, 2026</v>
       </c>
       <c r="L45" t="str">
-        <v>11 Aug 2026</v>
+        <v>Aug 11, 2026</v>
       </c>
       <c r="M45" t="str">
         <v>msokwhmdcolem</v>
@@ -2294,10 +2294,10 @@
         <v/>
       </c>
       <c r="K46" t="str">
-        <v>11 Aug 2026</v>
+        <v>Aug 11, 2026</v>
       </c>
       <c r="L46" t="str">
-        <v>11 Aug 2026</v>
+        <v>Aug 11, 2026</v>
       </c>
       <c r="M46" t="str">
         <v>msokwhmd3im81</v>
@@ -2335,10 +2335,10 @@
         <v/>
       </c>
       <c r="K47" t="str">
-        <v>11 Aug 2026</v>
+        <v>Aug 11, 2026</v>
       </c>
       <c r="L47" t="str">
-        <v>11 Aug 2026</v>
+        <v>Aug 11, 2026</v>
       </c>
       <c r="M47" t="str">
         <v>msokwhmdy3sam</v>
@@ -2376,10 +2376,10 @@
         <v/>
       </c>
       <c r="K48" t="str">
-        <v>11 Aug 2026</v>
+        <v>Aug 11, 2026</v>
       </c>
       <c r="L48" t="str">
-        <v>11 Aug 2026</v>
+        <v>Aug 11, 2026</v>
       </c>
       <c r="M48" t="str">
         <v>msokwhmdnrh8d</v>
@@ -2417,10 +2417,10 @@
         <v/>
       </c>
       <c r="K49" t="str">
-        <v>11 Aug 2026</v>
+        <v>Aug 11, 2026</v>
       </c>
       <c r="L49" t="str">
-        <v>11 Aug 2026</v>
+        <v>Aug 11, 2026</v>
       </c>
       <c r="M49" t="str">
         <v>msokwhmdjqudo</v>
@@ -2458,10 +2458,10 @@
         <v/>
       </c>
       <c r="K50" t="str">
-        <v>11 Aug 2026</v>
+        <v>Aug 11, 2026</v>
       </c>
       <c r="L50" t="str">
-        <v>11 Aug 2026</v>
+        <v>Aug 11, 2026</v>
       </c>
       <c r="M50" t="str">
         <v>msokwhmdew0dw</v>
@@ -2499,10 +2499,10 @@
         <v/>
       </c>
       <c r="K51" t="str">
-        <v>11 Aug 2026</v>
+        <v>Aug 11, 2026</v>
       </c>
       <c r="L51" t="str">
-        <v>11 Aug 2026</v>
+        <v>Aug 11, 2026</v>
       </c>
       <c r="M51" t="str">
         <v>msokwhmdul4ig</v>
@@ -2540,10 +2540,10 @@
         <v/>
       </c>
       <c r="K52" t="str">
-        <v>11 Aug 2026</v>
+        <v>Aug 11, 2026</v>
       </c>
       <c r="L52" t="str">
-        <v>11 Aug 2026</v>
+        <v>Aug 11, 2026</v>
       </c>
       <c r="M52" t="str">
         <v>msokwhmdgbas5</v>
@@ -2581,10 +2581,10 @@
         <v/>
       </c>
       <c r="K53" t="str">
-        <v>11 Aug 2026</v>
+        <v>Aug 11, 2026</v>
       </c>
       <c r="L53" t="str">
-        <v>11 Aug 2026</v>
+        <v>Aug 11, 2026</v>
       </c>
       <c r="M53" t="str">
         <v>msokxlxs06a9x</v>
@@ -2622,10 +2622,10 @@
         <v/>
       </c>
       <c r="K54" t="str">
-        <v>11 Aug 2026</v>
+        <v>Aug 11, 2026</v>
       </c>
       <c r="L54" t="str">
-        <v>11 Aug 2026</v>
+        <v>Aug 11, 2026</v>
       </c>
       <c r="M54" t="str">
         <v>msokxlxs42f77</v>
@@ -2663,10 +2663,10 @@
         <v/>
       </c>
       <c r="K55" t="str">
-        <v>11 Aug 2026</v>
+        <v>Aug 11, 2026</v>
       </c>
       <c r="L55" t="str">
-        <v>11 Aug 2026</v>
+        <v>Aug 11, 2026</v>
       </c>
       <c r="M55" t="str">
         <v>msokxlxs6xyeg</v>
@@ -2704,10 +2704,10 @@
         <v/>
       </c>
       <c r="K56" t="str">
-        <v>11 Aug 2026</v>
+        <v>Aug 11, 2026</v>
       </c>
       <c r="L56" t="str">
-        <v>11 Aug 2026</v>
+        <v>Aug 11, 2026</v>
       </c>
       <c r="M56" t="str">
         <v>msokxlxs7dltq</v>
@@ -2745,10 +2745,10 @@
         <v/>
       </c>
       <c r="K57" t="str">
-        <v>11 Aug 2026</v>
+        <v>Aug 11, 2026</v>
       </c>
       <c r="L57" t="str">
-        <v>11 Aug 2026</v>
+        <v>Aug 11, 2026</v>
       </c>
       <c r="M57" t="str">
         <v>msokxlxsgvc7b</v>
@@ -2786,10 +2786,10 @@
         <v/>
       </c>
       <c r="K58" t="str">
-        <v>11 Aug 2026</v>
+        <v>Aug 11, 2026</v>
       </c>
       <c r="L58" t="str">
-        <v>11 Aug 2026</v>
+        <v>Aug 11, 2026</v>
       </c>
       <c r="M58" t="str">
         <v>msokxlxsrox0v</v>
@@ -2827,10 +2827,10 @@
         <v/>
       </c>
       <c r="K59" t="str">
-        <v>11 Aug 2026</v>
+        <v>Aug 11, 2026</v>
       </c>
       <c r="L59" t="str">
-        <v>11 Aug 2026</v>
+        <v>Aug 11, 2026</v>
       </c>
       <c r="M59" t="str">
         <v>msokxlxsbwhdd</v>
@@ -2868,10 +2868,10 @@
         <v/>
       </c>
       <c r="K60" t="str">
-        <v>11 Aug 2026</v>
+        <v>Aug 11, 2026</v>
       </c>
       <c r="L60" t="str">
-        <v>11 Aug 2026</v>
+        <v>Aug 11, 2026</v>
       </c>
       <c r="M60" t="str">
         <v>msokxx7vw4unh</v>
@@ -2909,10 +2909,10 @@
         <v/>
       </c>
       <c r="K61" t="str">
-        <v>11 Aug 2026</v>
+        <v>Aug 11, 2026</v>
       </c>
       <c r="L61" t="str">
-        <v>11 Aug 2026</v>
+        <v>Aug 11, 2026</v>
       </c>
       <c r="M61" t="str">
         <v>msokxx7vcpo7d</v>
@@ -2950,10 +2950,10 @@
         <v/>
       </c>
       <c r="K62" t="str">
-        <v>11 Aug 2026</v>
+        <v>Aug 11, 2026</v>
       </c>
       <c r="L62" t="str">
-        <v>11 Aug 2026</v>
+        <v>Aug 11, 2026</v>
       </c>
       <c r="M62" t="str">
         <v>msokxx7vxd5a6</v>
@@ -2991,10 +2991,10 @@
         <v/>
       </c>
       <c r="K63" t="str">
-        <v>11 Aug 2026</v>
+        <v>Aug 11, 2026</v>
       </c>
       <c r="L63" t="str">
-        <v>11 Aug 2026</v>
+        <v>Aug 11, 2026</v>
       </c>
       <c r="M63" t="str">
         <v>msol0sqedwrwb</v>
@@ -3032,10 +3032,10 @@
         <v/>
       </c>
       <c r="K64" t="str">
-        <v>11 Aug 2026</v>
+        <v>Aug 11, 2026</v>
       </c>
       <c r="L64" t="str">
-        <v>11 Aug 2026</v>
+        <v>Aug 11, 2026</v>
       </c>
       <c r="M64" t="str">
         <v>msol0sqengvk7</v>
@@ -3073,10 +3073,10 @@
         <v/>
       </c>
       <c r="K65" t="str">
-        <v>11 Aug 2026</v>
+        <v>Aug 11, 2026</v>
       </c>
       <c r="L65" t="str">
-        <v>11 Aug 2026</v>
+        <v>Aug 11, 2026</v>
       </c>
       <c r="M65" t="str">
         <v>msol0sqeuws7d</v>
@@ -3114,10 +3114,10 @@
         <v/>
       </c>
       <c r="K66" t="str">
-        <v>11 Aug 2026</v>
+        <v>Aug 11, 2026</v>
       </c>
       <c r="L66" t="str">
-        <v>11 Aug 2026</v>
+        <v>Aug 11, 2026</v>
       </c>
       <c r="M66" t="str">
         <v>msol0sqekcfzc</v>
@@ -3155,10 +3155,10 @@
         <v/>
       </c>
       <c r="K67" t="str">
-        <v>11 Aug 2026</v>
+        <v>Aug 11, 2026</v>
       </c>
       <c r="L67" t="str">
-        <v>11 Aug 2026</v>
+        <v>Aug 11, 2026</v>
       </c>
       <c r="M67" t="str">
         <v>msol0sqemrzds</v>
@@ -3196,10 +3196,10 @@
         <v/>
       </c>
       <c r="K68" t="str">
-        <v>11 Aug 2026</v>
+        <v>Aug 11, 2026</v>
       </c>
       <c r="L68" t="str">
-        <v>11 Aug 2026</v>
+        <v>Aug 11, 2026</v>
       </c>
       <c r="M68" t="str">
         <v>msol0sqepq0ch</v>
@@ -3237,10 +3237,10 @@
         <v/>
       </c>
       <c r="K69" t="str">
-        <v>11 Aug 2026</v>
+        <v>Aug 11, 2026</v>
       </c>
       <c r="L69" t="str">
-        <v>11 Aug 2026</v>
+        <v>Aug 11, 2026</v>
       </c>
       <c r="M69" t="str">
         <v>msol0sqe12vt4</v>
@@ -3278,10 +3278,10 @@
         <v/>
       </c>
       <c r="K70" t="str">
-        <v>11 Aug 2026</v>
+        <v>Aug 11, 2026</v>
       </c>
       <c r="L70" t="str">
-        <v>11 Aug 2026</v>
+        <v>Aug 11, 2026</v>
       </c>
       <c r="M70" t="str">
         <v>msol0sqelotvw</v>
@@ -3319,10 +3319,10 @@
         <v/>
       </c>
       <c r="K71" t="str">
-        <v>11 Aug 2026</v>
+        <v>Aug 11, 2026</v>
       </c>
       <c r="L71" t="str">
-        <v>11 Aug 2026</v>
+        <v>Aug 11, 2026</v>
       </c>
       <c r="M71" t="str">
         <v>msol0sqe3ckax</v>
@@ -3360,10 +3360,10 @@
         <v/>
       </c>
       <c r="K72" t="str">
-        <v>11 Aug 2026</v>
+        <v>Aug 11, 2026</v>
       </c>
       <c r="L72" t="str">
-        <v>11 Aug 2026</v>
+        <v>Aug 11, 2026</v>
       </c>
       <c r="M72" t="str">
         <v>msol0sqe7neja</v>
@@ -3401,10 +3401,10 @@
         <v/>
       </c>
       <c r="K73" t="str">
-        <v>11 Aug 2026</v>
+        <v>Aug 11, 2026</v>
       </c>
       <c r="L73" t="str">
-        <v>11 Aug 2026</v>
+        <v>Aug 11, 2026</v>
       </c>
       <c r="M73" t="str">
         <v>msol0sqemccjp</v>
@@ -3442,10 +3442,10 @@
         <v/>
       </c>
       <c r="K74" t="str">
-        <v>11 Aug 2026</v>
+        <v>Aug 11, 2026</v>
       </c>
       <c r="L74" t="str">
-        <v>11 Aug 2026</v>
+        <v>Aug 11, 2026</v>
       </c>
       <c r="M74" t="str">
         <v>msol0sqei4fpl</v>
@@ -3483,10 +3483,10 @@
         <v/>
       </c>
       <c r="K75" t="str">
-        <v>11 Aug 2026</v>
+        <v>Aug 11, 2026</v>
       </c>
       <c r="L75" t="str">
-        <v>11 Aug 2026</v>
+        <v>Aug 11, 2026</v>
       </c>
       <c r="M75" t="str">
         <v>msol0sqe37ejp</v>
@@ -3524,10 +3524,10 @@
         <v/>
       </c>
       <c r="K76" t="str">
-        <v>11 Aug 2026</v>
+        <v>Aug 11, 2026</v>
       </c>
       <c r="L76" t="str">
-        <v>11 Aug 2026</v>
+        <v>Aug 11, 2026</v>
       </c>
       <c r="M76" t="str">
         <v>msol0sqe2tdno</v>
@@ -3565,10 +3565,10 @@
         <v/>
       </c>
       <c r="K77" t="str">
-        <v>11 Aug 2026</v>
+        <v>Aug 11, 2026</v>
       </c>
       <c r="L77" t="str">
-        <v>11 Aug 2026</v>
+        <v>Aug 11, 2026</v>
       </c>
       <c r="M77" t="str">
         <v>msol0sqe3wknl</v>
@@ -3606,10 +3606,10 @@
         <v/>
       </c>
       <c r="K78" t="str">
-        <v>11 Aug 2026</v>
+        <v>Aug 11, 2026</v>
       </c>
       <c r="L78" t="str">
-        <v>11 Aug 2026</v>
+        <v>Aug 11, 2026</v>
       </c>
       <c r="M78" t="str">
         <v>msol0sqejzchq</v>
@@ -3647,10 +3647,10 @@
         <v/>
       </c>
       <c r="K79" t="str">
-        <v>11 Aug 2026</v>
+        <v>Aug 11, 2026</v>
       </c>
       <c r="L79" t="str">
-        <v>11 Aug 2026</v>
+        <v>Aug 11, 2026</v>
       </c>
       <c r="M79" t="str">
         <v>msol0sqet2uhb</v>
@@ -3688,10 +3688,10 @@
         <v/>
       </c>
       <c r="K80" t="str">
-        <v>11 Aug 2026</v>
+        <v>Aug 11, 2026</v>
       </c>
       <c r="L80" t="str">
-        <v>11 Aug 2026</v>
+        <v>Aug 11, 2026</v>
       </c>
       <c r="M80" t="str">
         <v>msol0sqe5wsbz</v>
@@ -3729,10 +3729,10 @@
         <v/>
       </c>
       <c r="K81" t="str">
-        <v>11 Aug 2026</v>
+        <v>Aug 11, 2026</v>
       </c>
       <c r="L81" t="str">
-        <v>11 Aug 2026</v>
+        <v>Aug 11, 2026</v>
       </c>
       <c r="M81" t="str">
         <v>msol0sqezkuii</v>
@@ -3770,10 +3770,10 @@
         <v/>
       </c>
       <c r="K82" t="str">
-        <v>11 Aug 2026</v>
+        <v>Aug 11, 2026</v>
       </c>
       <c r="L82" t="str">
-        <v>11 Aug 2026</v>
+        <v>Aug 11, 2026</v>
       </c>
       <c r="M82" t="str">
         <v>msol0sqe4p67x</v>
@@ -3811,10 +3811,10 @@
         <v/>
       </c>
       <c r="K83" t="str">
-        <v>11 Aug 2026</v>
+        <v>Aug 11, 2026</v>
       </c>
       <c r="L83" t="str">
-        <v>11 Aug 2026</v>
+        <v>Aug 11, 2026</v>
       </c>
       <c r="M83" t="str">
         <v>msol0sqehxbfj</v>
@@ -3852,10 +3852,10 @@
         <v/>
       </c>
       <c r="K84" t="str">
-        <v>11 Aug 2026</v>
+        <v>Aug 11, 2026</v>
       </c>
       <c r="L84" t="str">
-        <v>11 Aug 2026</v>
+        <v>Aug 11, 2026</v>
       </c>
       <c r="M84" t="str">
         <v>msol0sqe6dg2v</v>
@@ -3893,10 +3893,10 @@
         <v/>
       </c>
       <c r="K85" t="str">
-        <v>11 Aug 2026</v>
+        <v>Aug 11, 2026</v>
       </c>
       <c r="L85" t="str">
-        <v>11 Aug 2026</v>
+        <v>Aug 11, 2026</v>
       </c>
       <c r="M85" t="str">
         <v>msol0sqewy04g</v>
@@ -3934,10 +3934,10 @@
         <v/>
       </c>
       <c r="K86" t="str">
-        <v>11 Aug 2026</v>
+        <v>Aug 11, 2026</v>
       </c>
       <c r="L86" t="str">
-        <v>11 Aug 2026</v>
+        <v>Aug 11, 2026</v>
       </c>
       <c r="M86" t="str">
         <v>msol0sqee580t</v>
@@ -3975,10 +3975,10 @@
         <v/>
       </c>
       <c r="K87" t="str">
-        <v>11 Aug 2026</v>
+        <v>Aug 11, 2026</v>
       </c>
       <c r="L87" t="str">
-        <v>11 Aug 2026</v>
+        <v>Aug 11, 2026</v>
       </c>
       <c r="M87" t="str">
         <v>msol0sqeiznyn</v>
@@ -4016,10 +4016,10 @@
         <v/>
       </c>
       <c r="K88" t="str">
-        <v>11 Aug 2026</v>
+        <v>Aug 11, 2026</v>
       </c>
       <c r="L88" t="str">
-        <v>11 Aug 2026</v>
+        <v>Aug 11, 2026</v>
       </c>
       <c r="M88" t="str">
         <v>msol0sqeohz5d</v>
@@ -4057,10 +4057,10 @@
         <v/>
       </c>
       <c r="K89" t="str">
-        <v>11 Aug 2026</v>
+        <v>Aug 11, 2026</v>
       </c>
       <c r="L89" t="str">
-        <v>11 Aug 2026</v>
+        <v>Aug 11, 2026</v>
       </c>
       <c r="M89" t="str">
         <v>msol0sqepq9bm</v>
@@ -4098,10 +4098,10 @@
         <v/>
       </c>
       <c r="K90" t="str">
-        <v>11 Aug 2026</v>
+        <v>Aug 11, 2026</v>
       </c>
       <c r="L90" t="str">
-        <v>11 Aug 2026</v>
+        <v>Aug 11, 2026</v>
       </c>
       <c r="M90" t="str">
         <v>msol0sqepn626</v>
@@ -4139,10 +4139,10 @@
         <v/>
       </c>
       <c r="K91" t="str">
-        <v>11 Aug 2026</v>
+        <v>Aug 11, 2026</v>
       </c>
       <c r="L91" t="str">
-        <v>11 Aug 2026</v>
+        <v>Aug 11, 2026</v>
       </c>
       <c r="M91" t="str">
         <v>msol0sqe28q4z</v>
@@ -4180,10 +4180,10 @@
         <v/>
       </c>
       <c r="K92" t="str">
-        <v>11 Aug 2026</v>
+        <v>Aug 11, 2026</v>
       </c>
       <c r="L92" t="str">
-        <v>11 Aug 2026</v>
+        <v>Aug 11, 2026</v>
       </c>
       <c r="M92" t="str">
         <v>msol0sqe56y72</v>
@@ -4221,10 +4221,10 @@
         <v/>
       </c>
       <c r="K93" t="str">
-        <v>11 Aug 2026</v>
+        <v>Aug 11, 2026</v>
       </c>
       <c r="L93" t="str">
-        <v>11 Aug 2026</v>
+        <v>Aug 11, 2026</v>
       </c>
       <c r="M93" t="str">
         <v>msol0sqeyukhl</v>
@@ -4262,10 +4262,10 @@
         <v/>
       </c>
       <c r="K94" t="str">
-        <v>11 Aug 2026</v>
+        <v>Aug 11, 2026</v>
       </c>
       <c r="L94" t="str">
-        <v>11 Aug 2026</v>
+        <v>Aug 11, 2026</v>
       </c>
       <c r="M94" t="str">
         <v>msol2k62oicjg</v>
@@ -4441,7 +4441,7 @@
     <col min="8" max="8" width="10.83203125" customWidth="1"/>
     <col min="9" max="9" width="10.83203125" customWidth="1"/>
     <col min="10" max="10" width="10.83203125" customWidth="1"/>
-    <col min="11" max="11" width="13.83203125" customWidth="1"/>
+    <col min="11" max="11" width="14.83203125" customWidth="1"/>
     <col min="12" max="12" width="18.83203125" customWidth="1"/>
     <col min="13" max="13" width="16.83203125" customWidth="1"/>
     <col min="14" max="14" width="16.83203125" customWidth="1"/>
@@ -4535,7 +4535,7 @@
         <v>53%</v>
       </c>
       <c r="K2" t="str">
-        <v>8 Aug 2026</v>
+        <v>Aug 8, 2026</v>
       </c>
       <c r="L2" t="str">
         <v>FALSE</v>
@@ -4588,7 +4588,7 @@
         <v>35%</v>
       </c>
       <c r="K3" t="str">
-        <v>8 Aug 2026</v>
+        <v>Aug 8, 2026</v>
       </c>
       <c r="L3" t="str">
         <v>FALSE</v>
@@ -4641,7 +4641,7 @@
         <v>0%</v>
       </c>
       <c r="K4" t="str">
-        <v>8 Aug 2026</v>
+        <v>Aug 8, 2026</v>
       </c>
       <c r="L4" t="str">
         <v>FALSE</v>
@@ -4694,7 +4694,7 @@
         <v>0%</v>
       </c>
       <c r="K5" t="str">
-        <v>11 Aug 2026</v>
+        <v>Aug 11, 2026</v>
       </c>
       <c r="L5" t="str">
         <v>TRUE</v>
@@ -4747,7 +4747,7 @@
         <v>0%</v>
       </c>
       <c r="K6" t="str">
-        <v>11 Aug 2026</v>
+        <v>Aug 11, 2026</v>
       </c>
       <c r="L6" t="str">
         <v>FALSE</v>
@@ -4800,7 +4800,7 @@
         <v>0%</v>
       </c>
       <c r="K7" t="str">
-        <v>11 Aug 2026</v>
+        <v>Aug 11, 2026</v>
       </c>
       <c r="L7" t="str">
         <v>FALSE</v>
@@ -4841,7 +4841,7 @@
     <col min="7" max="7" width="10.83203125" customWidth="1"/>
     <col min="8" max="8" width="10.83203125" customWidth="1"/>
     <col min="9" max="9" width="10.83203125" customWidth="1"/>
-    <col min="10" max="10" width="13.83203125" customWidth="1"/>
+    <col min="10" max="10" width="14.83203125" customWidth="1"/>
     <col min="11" max="11" width="15.83203125" customWidth="1"/>
   </cols>
   <sheetData>
@@ -4909,7 +4909,7 @@
         <v/>
       </c>
       <c r="J2" t="str">
-        <v>8 Aug 2026</v>
+        <v>Aug 8, 2026</v>
       </c>
       <c r="K2" t="str">
         <v>mskjvz8axp7bw</v>
@@ -4944,7 +4944,7 @@
         <v/>
       </c>
       <c r="J3" t="str">
-        <v>8 Aug 2026</v>
+        <v>Aug 8, 2026</v>
       </c>
       <c r="K3" t="str">
         <v>mskjw7zqqol4f</v>
@@ -4979,7 +4979,7 @@
         <v/>
       </c>
       <c r="J4" t="str">
-        <v>8 Aug 2026</v>
+        <v>Aug 8, 2026</v>
       </c>
       <c r="K4" t="str">
         <v>mskjwecwnzinb</v>
@@ -5014,7 +5014,7 @@
         <v/>
       </c>
       <c r="J5" t="str">
-        <v>8 Aug 2026</v>
+        <v>Aug 8, 2026</v>
       </c>
       <c r="K5" t="str">
         <v>mskjwjhp0kajz</v>
@@ -5049,7 +5049,7 @@
         <v/>
       </c>
       <c r="J6" t="str">
-        <v>8 Aug 2026</v>
+        <v>Aug 8, 2026</v>
       </c>
       <c r="K6" t="str">
         <v>mskjwo8nvlf63</v>
@@ -5084,7 +5084,7 @@
         <v/>
       </c>
       <c r="J7" t="str">
-        <v>8 Aug 2026</v>
+        <v>Aug 8, 2026</v>
       </c>
       <c r="K7" t="str">
         <v>mskjwtl16gyyh</v>
@@ -5127,7 +5127,7 @@
         <v/>
       </c>
       <c r="J8" t="str">
-        <v>8 Aug 2026</v>
+        <v>Aug 8, 2026</v>
       </c>
       <c r="K8" t="str">
         <v>mskk2136wm2x1</v>
@@ -5169,7 +5169,7 @@
         <v/>
       </c>
       <c r="J9" t="str">
-        <v>8 Aug 2026</v>
+        <v>Aug 8, 2026</v>
       </c>
       <c r="K9" t="str">
         <v>mskk2fgb7cnrq</v>
@@ -5220,7 +5220,7 @@
         <v/>
       </c>
       <c r="J10" t="str">
-        <v>8 Aug 2026</v>
+        <v>Aug 8, 2026</v>
       </c>
       <c r="K10" t="str">
         <v>mskk2w5rmle9n</v>
@@ -5255,7 +5255,7 @@
         <v/>
       </c>
       <c r="J11" t="str">
-        <v>10 Aug 2026</v>
+        <v>Aug 10, 2026</v>
       </c>
       <c r="K11" t="str">
         <v>msmnd1859wbzh</v>
@@ -5290,7 +5290,7 @@
         <v/>
       </c>
       <c r="J12" t="str">
-        <v>10 Aug 2026</v>
+        <v>Aug 10, 2026</v>
       </c>
       <c r="K12" t="str">
         <v>msmnd9ppyvwo0</v>
@@ -5325,7 +5325,7 @@
         <v/>
       </c>
       <c r="J13" t="str">
-        <v>10 Aug 2026</v>
+        <v>Aug 10, 2026</v>
       </c>
       <c r="K13" t="str">
         <v>msmndgl7h0wic</v>
@@ -5360,7 +5360,7 @@
         <v/>
       </c>
       <c r="J14" t="str">
-        <v>10 Aug 2026</v>
+        <v>Aug 10, 2026</v>
       </c>
       <c r="K14" t="str">
         <v>msmndnshe7g32</v>
@@ -5395,7 +5395,7 @@
         <v/>
       </c>
       <c r="J15" t="str">
-        <v>10 Aug 2026</v>
+        <v>Aug 10, 2026</v>
       </c>
       <c r="K15" t="str">
         <v>msmndu14o94q4</v>

</xml_diff>